<commit_message>
revert: chore: replace ACK circuit with TPS281C100 fault pin
</commit_message>
<xml_diff>
--- a/bom.xlsx
+++ b/bom.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="243">
   <si>
     <t xml:space="preserve">S3Main PCS BOM</t>
   </si>
@@ -134,7 +134,7 @@
     <t xml:space="preserve">Your Instructions / Notes</t>
   </si>
   <si>
-    <t xml:space="preserve">C1,C2,C3,C7,C8,C11,C18,C29,C30,C31</t>
+    <t xml:space="preserve">C1, C2, C3, C7, C8, C11, C18, C29, C30, C32</t>
   </si>
   <si>
     <t xml:space="preserve">Samsung Electro-Mechanics</t>
@@ -152,7 +152,7 @@
     <t xml:space="preserve">SMD</t>
   </si>
   <si>
-    <t xml:space="preserve">C4,C6,C19,C21,C22,C25,C26,C33</t>
+    <t xml:space="preserve">C4, C6, C19, C21, C22, C25, C26, C34</t>
   </si>
   <si>
     <t xml:space="preserve">Murata Electronics</t>
@@ -164,7 +164,7 @@
     <t xml:space="preserve">CAP CER 1000PF 100V C0G/NP0 0402</t>
   </si>
   <si>
-    <t xml:space="preserve">C5,C34,C35</t>
+    <t xml:space="preserve">C5, C35, C36</t>
   </si>
   <si>
     <t xml:space="preserve">GCM1555C1H221JA16D</t>
@@ -173,7 +173,7 @@
     <t xml:space="preserve">CAP CER 220PF 50V C0G/NP0 0402</t>
   </si>
   <si>
-    <t xml:space="preserve">C9,C10</t>
+    <t xml:space="preserve">C9, C10</t>
   </si>
   <si>
     <t xml:space="preserve">GCM1555C1H101JA16D</t>
@@ -182,7 +182,7 @@
     <t xml:space="preserve">CAP CER 100PF 50V C0G/NP0 0402</t>
   </si>
   <si>
-    <t xml:space="preserve">C12,C20,C27</t>
+    <t xml:space="preserve">C12, C20, C27</t>
   </si>
   <si>
     <t xml:space="preserve">Cornell Dubilier Knowles</t>
@@ -218,7 +218,7 @@
     <t xml:space="preserve">CAP CER 10UF 50V X7R 1206</t>
   </si>
   <si>
-    <t xml:space="preserve">C15,C16,C17,C23,C24</t>
+    <t xml:space="preserve">C15, C16, C17, C23, C24</t>
   </si>
   <si>
     <t xml:space="preserve">CL31B105KCHVPJE</t>
@@ -236,7 +236,16 @@
     <t xml:space="preserve">CAP CER 4.7UF 50V X7R 1206</t>
   </si>
   <si>
-    <t xml:space="preserve">C32,C36</t>
+    <t xml:space="preserve">C31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GRT3195C2A103JA02D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAP CER 10000PF 100V C0G 1206</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C33, C37</t>
   </si>
   <si>
     <t xml:space="preserve">TDK Corporation</t>
@@ -248,7 +257,7 @@
     <t xml:space="preserve">CAP CER 47UF 6.3V X7S 1206</t>
   </si>
   <si>
-    <t xml:space="preserve">D1,D2,D3,D7,D8,D11,D13,D14,D15,D17</t>
+    <t xml:space="preserve">D1, D2, D3, D7, D8, D11, D13, D16, D17, D19</t>
   </si>
   <si>
     <t xml:space="preserve">onsemi</t>
@@ -335,7 +344,22 @@
     <t xml:space="preserve">TVS DIODE 30VWM 47.5VC ESC</t>
   </si>
   <si>
-    <t xml:space="preserve">D16</t>
+    <t xml:space="preserve">D14, D15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Micro Commercial Co</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B5819W-TP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIODE SCHOTTKY 40V 1A SOD123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOD-123</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D18</t>
   </si>
   <si>
     <t xml:space="preserve">Diodes Incorporated</t>
@@ -416,7 +440,7 @@
     <t xml:space="preserve">0805</t>
   </si>
   <si>
-    <t xml:space="preserve">Q1,Q6</t>
+    <t xml:space="preserve">Q1, Q6</t>
   </si>
   <si>
     <t xml:space="preserve">Rohm Semiconductor</t>
@@ -443,7 +467,7 @@
     <t xml:space="preserve">SOT-363</t>
   </si>
   <si>
-    <t xml:space="preserve">Q3,Q4,Q5,Q7,Q8</t>
+    <t xml:space="preserve">Q3, Q4, Q5, Q7, Q8</t>
   </si>
   <si>
     <t xml:space="preserve">Vishay Siliconix</t>
@@ -461,6 +485,15 @@
     <t xml:space="preserve">Q9</t>
   </si>
   <si>
+    <t xml:space="preserve">BSS138</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MOSFET N-CH 50V 220MA SOT23-3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q10</t>
+  </si>
+  <si>
     <t xml:space="preserve">ANBON SEMICONDUCTOR (INT'L) LIMITED</t>
   </si>
   <si>
@@ -473,7 +506,7 @@
     <t xml:space="preserve">SOT-23</t>
   </si>
   <si>
-    <t xml:space="preserve">R1,R8,R18,R20,R35,R36,R37,R44,R49</t>
+    <t xml:space="preserve">R1, R8, R18, R20, R34, R35, R36, R43, R48, R50</t>
   </si>
   <si>
     <t xml:space="preserve">YAGEO</t>
@@ -485,7 +518,7 @@
     <t xml:space="preserve">RES 10K OHM 1% 1/16W 0402</t>
   </si>
   <si>
-    <t xml:space="preserve">R2,R3,R4,R5</t>
+    <t xml:space="preserve">R2, R3, R4, R5</t>
   </si>
   <si>
     <t xml:space="preserve">RC0402FR-0722KL</t>
@@ -494,7 +527,7 @@
     <t xml:space="preserve">RES 22K OHM 1% 1/16W 0402</t>
   </si>
   <si>
-    <t xml:space="preserve">R6,R7,R31</t>
+    <t xml:space="preserve">R6, R7, R31, R49</t>
   </si>
   <si>
     <t xml:space="preserve">RC0402FR-074K7L</t>
@@ -515,7 +548,7 @@
     <t xml:space="preserve">RES SMD 2.2 OHM 1% 1/2W 0805</t>
   </si>
   <si>
-    <t xml:space="preserve">R10,R11,R14,R32,R46</t>
+    <t xml:space="preserve">R10, R11, R14, R32, R45, R51</t>
   </si>
   <si>
     <t xml:space="preserve">RC0402FR-071KL</t>
@@ -524,7 +557,7 @@
     <t xml:space="preserve">RES 1K OHM 1% 1/16W 0402</t>
   </si>
   <si>
-    <t xml:space="preserve">R12,R13,R22,R26,R27</t>
+    <t xml:space="preserve">R12, R13, R22, R26, R27</t>
   </si>
   <si>
     <t xml:space="preserve">RC0402FR-073K3L</t>
@@ -533,7 +566,7 @@
     <t xml:space="preserve">RES 3.3K OHM 1% 1/16W 0402</t>
   </si>
   <si>
-    <t xml:space="preserve">R15,R16,R50,R51</t>
+    <t xml:space="preserve">R15, R16, R52, R53</t>
   </si>
   <si>
     <t xml:space="preserve">RC0402FR-0733RL</t>
@@ -551,7 +584,7 @@
     <t xml:space="preserve">RES 220 OHM 1% 1/16W 0402</t>
   </si>
   <si>
-    <t xml:space="preserve">R19,R34</t>
+    <t xml:space="preserve">R19, R54</t>
   </si>
   <si>
     <t xml:space="preserve">DNP</t>
@@ -575,7 +608,7 @@
     <t xml:space="preserve">RES 562 OHM 1% 1/16W 0402</t>
   </si>
   <si>
-    <t xml:space="preserve">R24,R25</t>
+    <t xml:space="preserve">R24, R25</t>
   </si>
   <si>
     <t xml:space="preserve">R28</t>
@@ -587,7 +620,7 @@
     <t xml:space="preserve">RES 422 OHM 1% 1/16W 0402</t>
   </si>
   <si>
-    <t xml:space="preserve">R29,R30,R47,R48</t>
+    <t xml:space="preserve">R29, R30, R46, R47</t>
   </si>
   <si>
     <t xml:space="preserve">RC0402FR-0747RL</t>
@@ -605,7 +638,7 @@
     <t xml:space="preserve">RES 180 OHM 1% 1/16W 0402</t>
   </si>
   <si>
-    <t xml:space="preserve">R38,R45</t>
+    <t xml:space="preserve">R37, R44</t>
   </si>
   <si>
     <t xml:space="preserve">RC0402FR-0714K3L</t>
@@ -614,25 +647,25 @@
     <t xml:space="preserve">RES 14.3K OHM 1% 1/16W 0402</t>
   </si>
   <si>
+    <t xml:space="preserve">R38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC0402FR-07470RL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RES 470 OHM 1% 1/16W 0402</t>
+  </si>
+  <si>
     <t xml:space="preserve">R39</t>
   </si>
   <si>
-    <t xml:space="preserve">RC0402FR-07470RL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RES 470 OHM 1% 1/16W 0402</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R40</t>
-  </si>
-  <si>
     <t xml:space="preserve">RC0402FR-0718K7L</t>
   </si>
   <si>
     <t xml:space="preserve">RES 18.7K OHM 1% 1/16W 0402</t>
   </si>
   <si>
-    <t xml:space="preserve">R41,R42</t>
+    <t xml:space="preserve">R40, R41</t>
   </si>
   <si>
     <t xml:space="preserve">RC0402FR-075K1L</t>
@@ -641,7 +674,7 @@
     <t xml:space="preserve">RES 5.1K OHM 1% 1/16W 0402</t>
   </si>
   <si>
-    <t xml:space="preserve">R43</t>
+    <t xml:space="preserve">R42</t>
   </si>
   <si>
     <t xml:space="preserve">RC0402FR-0739KL</t>
@@ -650,7 +683,7 @@
     <t xml:space="preserve">RES 39K OHM 1% 1/16W 0402</t>
   </si>
   <si>
-    <t xml:space="preserve">R52</t>
+    <t xml:space="preserve">R55</t>
   </si>
   <si>
     <t xml:space="preserve">Panasonic Electronic Components</t>
@@ -1072,13 +1105,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>649440</xdr:colOff>
+      <xdr:colOff>649800</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>141840</xdr:rowOff>
+      <xdr:rowOff>142200</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="图片 1" descr="pcbway-400x400.jpg"/>
+        <xdr:cNvPr id="0" name="图片 1" descr="pcbway-400x400.jpg"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1088,7 +1121,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="9360" y="211680"/>
-          <a:ext cx="1360080" cy="358920"/>
+          <a:ext cx="1360440" cy="359280"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1531,16 +1564,16 @@
         <v>44</v>
       </c>
       <c r="C16" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D16" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E16" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="E16" s="7" t="s">
+      <c r="F16" s="8" t="s">
         <v>46</v>
-      </c>
-      <c r="F16" s="8" t="s">
-        <v>47</v>
       </c>
       <c r="G16" s="9" t="s">
         <v>34</v>
@@ -1555,22 +1588,22 @@
         <v>11</v>
       </c>
       <c r="B17" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C17" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="C17" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="D17" s="7" t="s">
+      <c r="E17" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="F17" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="F17" s="8" t="s">
-        <v>51</v>
-      </c>
       <c r="G17" s="9" t="s">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="H17" s="10" t="s">
         <v>15</v>
@@ -1582,22 +1615,22 @@
         <v>12</v>
       </c>
       <c r="B18" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="E18" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="C18" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="7" t="s">
+      <c r="F18" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="G18" s="9" t="s">
         <v>55</v>
-      </c>
-      <c r="F18" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="G18" s="9" t="s">
-        <v>14</v>
       </c>
       <c r="H18" s="10" t="s">
         <v>15</v>
@@ -1609,13 +1642,13 @@
         <v>13</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C19" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="E19" s="7" t="s">
         <v>58</v>
@@ -1642,7 +1675,7 @@
         <v>1</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="E20" s="7" t="s">
         <v>61</v>
@@ -1669,16 +1702,16 @@
         <v>1</v>
       </c>
       <c r="D21" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="E21" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="E21" s="7" t="s">
+      <c r="F21" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="F21" s="8" t="s">
-        <v>66</v>
-      </c>
       <c r="G21" s="9" t="s">
-        <v>67</v>
+        <v>14</v>
       </c>
       <c r="H21" s="10" t="s">
         <v>15</v>
@@ -1690,22 +1723,22 @@
         <v>16</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C22" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D22" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="F22" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="E22" s="7" t="s">
+      <c r="G22" s="9" t="s">
         <v>70</v>
-      </c>
-      <c r="F22" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="G22" s="9" t="s">
-        <v>72</v>
       </c>
       <c r="H22" s="10" t="s">
         <v>15</v>
@@ -1717,22 +1750,22 @@
         <v>17</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C23" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D23" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="F23" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="G23" s="9" t="s">
         <v>75</v>
-      </c>
-      <c r="F23" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="G23" s="9" t="s">
-        <v>52</v>
       </c>
       <c r="H23" s="10" t="s">
         <v>15</v>
@@ -1744,22 +1777,22 @@
         <v>18</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C24" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D24" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="E24" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="E24" s="7" t="s">
+      <c r="F24" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="F24" s="7" t="s">
-        <v>80</v>
-      </c>
       <c r="G24" s="9" t="s">
-        <v>81</v>
+        <v>55</v>
       </c>
       <c r="H24" s="10" t="s">
         <v>15</v>
@@ -1771,23 +1804,25 @@
         <v>19</v>
       </c>
       <c r="B25" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="E25" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="C25" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" s="7" t="s">
+      <c r="F25" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="E25" s="7" t="n">
-        <v>1844210</v>
-      </c>
-      <c r="F25" s="8" t="s">
+      <c r="G25" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="G25" s="9"/>
       <c r="H25" s="10" t="s">
-        <v>85</v>
+        <v>15</v>
       </c>
       <c r="I25" s="10"/>
     </row>
@@ -1796,21 +1831,23 @@
         <v>20</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C26" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D26" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="E26" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="E26" s="7" t="s">
+      <c r="F26" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="F26" s="8" t="s">
+      <c r="G26" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="G26" s="9"/>
       <c r="H26" s="10" t="s">
         <v>15</v>
       </c>
@@ -1827,17 +1864,17 @@
         <v>1</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>1836189</v>
+        <v>1844210</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G27" s="9"/>
       <c r="H27" s="10" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="I27" s="10"/>
     </row>
@@ -1846,19 +1883,19 @@
         <v>22</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="C28" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G28" s="9"/>
       <c r="H28" s="10" t="s">
@@ -1871,23 +1908,23 @@
         <v>23</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C29" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="E29" s="7" t="s">
-        <v>98</v>
+        <v>91</v>
+      </c>
+      <c r="E29" s="7" t="n">
+        <v>1836189</v>
       </c>
       <c r="F29" s="8" t="s">
         <v>99</v>
       </c>
       <c r="G29" s="9"/>
       <c r="H29" s="10" t="s">
-        <v>15</v>
+        <v>93</v>
       </c>
       <c r="I29" s="10"/>
     </row>
@@ -1902,17 +1939,15 @@
         <v>1</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>17</v>
+        <v>101</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F30" s="8" t="s">
-        <v>102</v>
-      </c>
-      <c r="G30" s="9" t="s">
         <v>103</v>
       </c>
+      <c r="G30" s="9"/>
       <c r="H30" s="10" t="s">
         <v>15</v>
       </c>
@@ -1926,7 +1961,7 @@
         <v>104</v>
       </c>
       <c r="C31" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D31" s="7" t="s">
         <v>105</v>
@@ -1934,12 +1969,10 @@
       <c r="E31" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="F31" s="7" t="s">
+      <c r="F31" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="G31" s="9" t="s">
-        <v>108</v>
-      </c>
+      <c r="G31" s="9"/>
       <c r="H31" s="10" t="s">
         <v>15</v>
       </c>
@@ -1950,22 +1983,22 @@
         <v>26</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C32" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D32" s="7" t="s">
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="E32" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="F32" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="F32" s="7" t="s">
+      <c r="G32" s="9" t="s">
         <v>111</v>
-      </c>
-      <c r="G32" s="9" t="s">
-        <v>112</v>
       </c>
       <c r="H32" s="10" t="s">
         <v>15</v>
@@ -1977,22 +2010,22 @@
         <v>27</v>
       </c>
       <c r="B33" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="C33" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D33" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="C33" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="D33" s="7" t="s">
+      <c r="E33" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="E33" s="7" t="s">
+      <c r="F33" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="F33" s="8" t="s">
+      <c r="G33" s="9" t="s">
         <v>116</v>
-      </c>
-      <c r="G33" s="9" t="s">
-        <v>117</v>
       </c>
       <c r="H33" s="10" t="s">
         <v>15</v>
@@ -2004,22 +2037,22 @@
         <v>28</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C34" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D34" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="E34" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="F34" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="E34" s="7" t="s">
+      <c r="G34" s="9" t="s">
         <v>120</v>
-      </c>
-      <c r="F34" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="G34" s="9" t="s">
-        <v>122</v>
       </c>
       <c r="H34" s="10" t="s">
         <v>15</v>
@@ -2031,22 +2064,22 @@
         <v>29</v>
       </c>
       <c r="B35" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="C35" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="E35" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="C35" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="D35" s="7" t="s">
+      <c r="F35" s="8" t="s">
         <v>124</v>
       </c>
-      <c r="E35" s="7" t="s">
+      <c r="G35" s="9" t="s">
         <v>125</v>
-      </c>
-      <c r="F35" s="7" t="s">
-        <v>126</v>
-      </c>
-      <c r="G35" s="9" t="s">
-        <v>14</v>
       </c>
       <c r="H35" s="10" t="s">
         <v>15</v>
@@ -2058,22 +2091,22 @@
         <v>30</v>
       </c>
       <c r="B36" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="C36" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="E36" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="C36" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="D36" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="E36" s="7" t="s">
+      <c r="F36" s="7" t="s">
         <v>128</v>
       </c>
-      <c r="F36" s="7" t="s">
-        <v>129</v>
-      </c>
       <c r="G36" s="9" t="s">
-        <v>14</v>
+        <v>70</v>
       </c>
       <c r="H36" s="10" t="s">
         <v>15</v>
@@ -2085,13 +2118,13 @@
         <v>31</v>
       </c>
       <c r="B37" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="C37" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="7" t="s">
         <v>130</v>
-      </c>
-      <c r="C37" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="D37" s="7" t="s">
-        <v>124</v>
       </c>
       <c r="E37" s="7" t="s">
         <v>131</v>
@@ -2100,7 +2133,7 @@
         <v>132</v>
       </c>
       <c r="G37" s="9" t="s">
-        <v>14</v>
+        <v>133</v>
       </c>
       <c r="H37" s="10" t="s">
         <v>15</v>
@@ -2112,22 +2145,22 @@
         <v>32</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C38" s="6" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E38" s="7" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F38" s="7" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G38" s="9" t="s">
-        <v>103</v>
+        <v>14</v>
       </c>
       <c r="H38" s="10" t="s">
         <v>15</v>
@@ -2139,19 +2172,19 @@
         <v>33</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C39" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="E39" s="7" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G39" s="9" t="s">
         <v>14</v>
@@ -2166,19 +2199,19 @@
         <v>34</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C40" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F40" s="7" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="G40" s="9" t="s">
         <v>14</v>
@@ -2193,22 +2226,22 @@
         <v>35</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C41" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="E41" s="7" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F41" s="7" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G41" s="9" t="s">
-        <v>14</v>
+        <v>111</v>
       </c>
       <c r="H41" s="10" t="s">
         <v>15</v>
@@ -2220,19 +2253,19 @@
         <v>36</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C42" s="6" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="E42" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="F42" s="8" t="s">
-        <v>148</v>
+        <v>149</v>
+      </c>
+      <c r="F42" s="7" t="s">
+        <v>150</v>
       </c>
       <c r="G42" s="9" t="s">
         <v>14</v>
@@ -2247,19 +2280,25 @@
         <v>37</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C43" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D43" s="7"/>
-      <c r="E43" s="7"/>
-      <c r="F43" s="8"/>
-      <c r="G43" s="10" t="s">
-        <v>150</v>
+        <v>5</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="E43" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="F43" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="G43" s="9" t="s">
+        <v>14</v>
       </c>
       <c r="H43" s="10" t="s">
-        <v>150</v>
+        <v>15</v>
       </c>
       <c r="I43" s="10"/>
     </row>
@@ -2268,19 +2307,19 @@
         <v>38</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="C44" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D44" s="7" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="E44" s="7" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="F44" s="7" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="G44" s="9" t="s">
         <v>14</v>
@@ -2295,19 +2334,19 @@
         <v>39</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="C45" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D45" s="7" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="E45" s="7" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="F45" s="8" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="G45" s="9" t="s">
         <v>14</v>
@@ -2322,7 +2361,7 @@
         <v>40</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C46" s="6" t="n">
         <v>2</v>
@@ -2331,10 +2370,10 @@
       <c r="E46" s="7"/>
       <c r="F46" s="8"/>
       <c r="G46" s="10" t="s">
-        <v>150</v>
+        <v>161</v>
       </c>
       <c r="H46" s="10" t="s">
-        <v>150</v>
+        <v>161</v>
       </c>
       <c r="I46" s="10"/>
     </row>
@@ -2343,19 +2382,19 @@
         <v>41</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="C47" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="E47" s="7" t="s">
-        <v>159</v>
-      </c>
-      <c r="F47" s="8" t="s">
-        <v>160</v>
+        <v>163</v>
+      </c>
+      <c r="F47" s="7" t="s">
+        <v>164</v>
       </c>
       <c r="G47" s="9" t="s">
         <v>14</v>
@@ -2370,19 +2409,19 @@
         <v>42</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="C48" s="6" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D48" s="7" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="E48" s="7" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="F48" s="8" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="G48" s="9" t="s">
         <v>14</v>
@@ -2397,25 +2436,19 @@
         <v>43</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="C49" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D49" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="E49" s="7" t="s">
-        <v>165</v>
-      </c>
-      <c r="F49" s="8" t="s">
-        <v>166</v>
-      </c>
-      <c r="G49" s="9" t="s">
-        <v>14</v>
+        <v>2</v>
+      </c>
+      <c r="D49" s="7"/>
+      <c r="E49" s="7"/>
+      <c r="F49" s="8"/>
+      <c r="G49" s="10" t="s">
+        <v>161</v>
       </c>
       <c r="H49" s="10" t="s">
-        <v>15</v>
+        <v>161</v>
       </c>
       <c r="I49" s="10"/>
     </row>
@@ -2424,19 +2457,19 @@
         <v>44</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C50" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D50" s="7" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="E50" s="7" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="F50" s="8" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="G50" s="9" t="s">
         <v>14</v>
@@ -2451,19 +2484,19 @@
         <v>45</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C51" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D51" s="7" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="E51" s="7" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="F51" s="8" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="G51" s="9" t="s">
         <v>14</v>
@@ -2478,19 +2511,19 @@
         <v>46</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C52" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D52" s="7" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="E52" s="7" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="F52" s="8" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="G52" s="9" t="s">
         <v>14</v>
@@ -2505,19 +2538,19 @@
         <v>47</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C53" s="6" t="n">
         <v>2</v>
       </c>
       <c r="D53" s="7" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="E53" s="7" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F53" s="8" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="G53" s="9" t="s">
         <v>14</v>
@@ -2532,19 +2565,19 @@
         <v>48</v>
       </c>
       <c r="B54" s="7" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C54" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D54" s="7" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="E54" s="7" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="F54" s="8" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="G54" s="9" t="s">
         <v>14</v>
@@ -2559,19 +2592,19 @@
         <v>49</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C55" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D55" s="7" t="s">
-        <v>183</v>
+        <v>135</v>
       </c>
       <c r="E55" s="7" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F55" s="8" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G55" s="9" t="s">
         <v>14</v>
@@ -2586,22 +2619,22 @@
         <v>50</v>
       </c>
       <c r="B56" s="7" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C56" s="6" t="n">
         <v>2</v>
       </c>
       <c r="D56" s="7" t="s">
-        <v>183</v>
+        <v>135</v>
       </c>
       <c r="E56" s="7" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F56" s="8" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="G56" s="9" t="s">
-        <v>189</v>
+        <v>14</v>
       </c>
       <c r="H56" s="10" t="s">
         <v>15</v>
@@ -2619,16 +2652,16 @@
         <v>1</v>
       </c>
       <c r="D57" s="7" t="s">
-        <v>49</v>
+        <v>135</v>
       </c>
       <c r="E57" s="7" t="s">
         <v>191</v>
       </c>
-      <c r="F57" s="7" t="s">
+      <c r="F57" s="8" t="s">
         <v>192</v>
       </c>
       <c r="G57" s="9" t="s">
-        <v>193</v>
+        <v>14</v>
       </c>
       <c r="H57" s="10" t="s">
         <v>15</v>
@@ -2640,22 +2673,22 @@
         <v>52</v>
       </c>
       <c r="B58" s="7" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C58" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D58" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="E58" s="7" t="s">
         <v>195</v>
       </c>
-      <c r="E58" s="7" t="s">
+      <c r="F58" s="8" t="s">
         <v>196</v>
       </c>
-      <c r="F58" s="8" t="s">
-        <v>197</v>
-      </c>
       <c r="G58" s="9" t="s">
-        <v>198</v>
+        <v>14</v>
       </c>
       <c r="H58" s="10" t="s">
         <v>15</v>
@@ -2667,22 +2700,22 @@
         <v>53</v>
       </c>
       <c r="B59" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="C59" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D59" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="E59" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="F59" s="8" t="s">
         <v>199</v>
       </c>
-      <c r="C59" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D59" s="7" t="s">
+      <c r="G59" s="9" t="s">
         <v>200</v>
-      </c>
-      <c r="E59" s="7" t="s">
-        <v>201</v>
-      </c>
-      <c r="F59" s="8" t="s">
-        <v>202</v>
-      </c>
-      <c r="G59" s="9" t="s">
-        <v>203</v>
       </c>
       <c r="H59" s="10" t="s">
         <v>15</v>
@@ -2694,21 +2727,23 @@
         <v>54</v>
       </c>
       <c r="B60" s="7" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C60" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D60" s="7" t="s">
-        <v>205</v>
+        <v>52</v>
       </c>
       <c r="E60" s="7" t="s">
-        <v>206</v>
-      </c>
-      <c r="F60" s="8" t="s">
-        <v>207</v>
-      </c>
-      <c r="G60" s="9"/>
+        <v>202</v>
+      </c>
+      <c r="F60" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="G60" s="9" t="s">
+        <v>204</v>
+      </c>
       <c r="H60" s="10" t="s">
         <v>15</v>
       </c>
@@ -2719,22 +2754,22 @@
         <v>55</v>
       </c>
       <c r="B61" s="7" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="C61" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D61" s="7" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="E61" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="F61" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="G61" s="9" t="s">
         <v>209</v>
-      </c>
-      <c r="F61" s="7" t="s">
-        <v>210</v>
-      </c>
-      <c r="G61" s="9" t="s">
-        <v>211</v>
       </c>
       <c r="H61" s="10" t="s">
         <v>15</v>
@@ -2746,22 +2781,22 @@
         <v>56</v>
       </c>
       <c r="B62" s="7" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C62" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D62" s="7" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="E62" s="7" t="s">
+        <v>212</v>
+      </c>
+      <c r="F62" s="8" t="s">
         <v>213</v>
       </c>
-      <c r="F62" s="8" t="s">
+      <c r="G62" s="9" t="s">
         <v>214</v>
-      </c>
-      <c r="G62" s="9" t="s">
-        <v>215</v>
       </c>
       <c r="H62" s="10" t="s">
         <v>15</v>
@@ -2773,13 +2808,13 @@
         <v>57</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C63" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D63" s="7" t="s">
-        <v>78</v>
+        <v>216</v>
       </c>
       <c r="E63" s="7" t="s">
         <v>217</v>
@@ -2787,9 +2822,7 @@
       <c r="F63" s="8" t="s">
         <v>218</v>
       </c>
-      <c r="G63" s="9" t="s">
-        <v>72</v>
-      </c>
+      <c r="G63" s="9"/>
       <c r="H63" s="10" t="s">
         <v>15</v>
       </c>
@@ -2806,12 +2839,12 @@
         <v>1</v>
       </c>
       <c r="D64" s="7" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="E64" s="7" t="s">
         <v>220</v>
       </c>
-      <c r="F64" s="12" t="s">
+      <c r="F64" s="7" t="s">
         <v>221</v>
       </c>
       <c r="G64" s="9" t="s">
@@ -2833,7 +2866,7 @@
         <v>1</v>
       </c>
       <c r="D65" s="7" t="s">
-        <v>78</v>
+        <v>211</v>
       </c>
       <c r="E65" s="7" t="s">
         <v>224</v>
@@ -2860,1055 +2893,1133 @@
         <v>1</v>
       </c>
       <c r="D66" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="E66" s="7" t="s">
         <v>228</v>
       </c>
-      <c r="E66" s="7" t="s">
+      <c r="F66" s="8" t="s">
         <v>229</v>
       </c>
-      <c r="F66" s="8" t="s">
+      <c r="G66" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="H66" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="I66" s="10"/>
+    </row>
+    <row r="67" s="11" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="6" t="n">
+        <v>61</v>
+      </c>
+      <c r="B67" s="7" t="s">
         <v>230</v>
       </c>
-      <c r="G66" s="9" t="s">
+      <c r="C67" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="E67" s="7" t="s">
         <v>231</v>
       </c>
-      <c r="H66" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="I66" s="10"/>
-    </row>
-    <row r="67" s="11" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="68" s="11" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="69" s="11" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="F67" s="12" t="s">
+        <v>232</v>
+      </c>
+      <c r="G67" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="H67" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="I67" s="10"/>
+    </row>
+    <row r="68" s="11" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="6" t="n">
+        <v>62</v>
+      </c>
+      <c r="B68" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="C68" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D68" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="E68" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="F68" s="8" t="s">
+        <v>236</v>
+      </c>
+      <c r="G68" s="9" t="s">
+        <v>237</v>
+      </c>
+      <c r="H68" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="I68" s="10"/>
+    </row>
+    <row r="69" s="11" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="6" t="n">
+        <v>63</v>
+      </c>
+      <c r="B69" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="C69" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D69" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="E69" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="F69" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="G69" s="9" t="s">
+        <v>242</v>
+      </c>
+      <c r="H69" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="I69" s="10"/>
+    </row>
     <row r="70" s="11" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="71" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="11"/>
-      <c r="B71" s="11"/>
-      <c r="C71" s="11"/>
-      <c r="D71" s="11"/>
-      <c r="E71" s="11"/>
-      <c r="F71" s="11"/>
-      <c r="G71" s="11"/>
-      <c r="H71" s="11"/>
-      <c r="I71" s="11"/>
-      <c r="J71" s="11"/>
-      <c r="K71" s="11"/>
-      <c r="L71" s="11"/>
-      <c r="M71" s="11"/>
-      <c r="N71" s="11"/>
-      <c r="O71" s="11"/>
-      <c r="P71" s="11"/>
-      <c r="Q71" s="11"/>
-      <c r="R71" s="11"/>
-      <c r="S71" s="11"/>
-      <c r="T71" s="11"/>
-      <c r="U71" s="11"/>
-      <c r="V71" s="11"/>
-      <c r="W71" s="11"/>
-      <c r="X71" s="11"/>
-      <c r="Y71" s="11"/>
-      <c r="Z71" s="11"/>
-      <c r="AA71" s="11"/>
-      <c r="AB71" s="11"/>
-      <c r="AC71" s="11"/>
-      <c r="AD71" s="11"/>
-      <c r="AE71" s="11"/>
-      <c r="AF71" s="11"/>
-      <c r="AG71" s="11"/>
-      <c r="AH71" s="11"/>
-      <c r="AI71" s="11"/>
-      <c r="AJ71" s="11"/>
-      <c r="AK71" s="11"/>
-      <c r="AL71" s="11"/>
-      <c r="AM71" s="11"/>
-      <c r="AN71" s="11"/>
-      <c r="AO71" s="11"/>
-      <c r="AP71" s="11"/>
-      <c r="AQ71" s="11"/>
-      <c r="AR71" s="11"/>
-      <c r="AS71" s="11"/>
-      <c r="AT71" s="11"/>
-      <c r="AU71" s="11"/>
-      <c r="AV71" s="11"/>
-      <c r="AW71" s="11"/>
-      <c r="AX71" s="11"/>
-      <c r="AY71" s="11"/>
-      <c r="AZ71" s="11"/>
-      <c r="BA71" s="11"/>
-      <c r="BB71" s="11"/>
-      <c r="BC71" s="11"/>
-      <c r="BD71" s="11"/>
-      <c r="BE71" s="11"/>
-      <c r="BF71" s="11"/>
-      <c r="BG71" s="11"/>
-      <c r="BH71" s="11"/>
-      <c r="BI71" s="11"/>
-      <c r="BJ71" s="11"/>
-      <c r="BK71" s="11"/>
-      <c r="BL71" s="11"/>
-      <c r="BM71" s="11"/>
-      <c r="BN71" s="11"/>
-      <c r="BO71" s="11"/>
-      <c r="BP71" s="11"/>
-      <c r="BQ71" s="11"/>
-      <c r="BR71" s="11"/>
-      <c r="BS71" s="11"/>
-      <c r="BT71" s="11"/>
-      <c r="BU71" s="11"/>
-      <c r="BV71" s="11"/>
-      <c r="BW71" s="11"/>
-      <c r="BX71" s="11"/>
-      <c r="BY71" s="11"/>
-      <c r="BZ71" s="11"/>
-      <c r="CA71" s="11"/>
-      <c r="CB71" s="11"/>
-      <c r="CC71" s="11"/>
-      <c r="CD71" s="11"/>
-      <c r="CE71" s="11"/>
-      <c r="CF71" s="11"/>
-      <c r="CG71" s="11"/>
-      <c r="CH71" s="11"/>
-      <c r="CI71" s="11"/>
-      <c r="CJ71" s="11"/>
-      <c r="CK71" s="11"/>
-      <c r="CL71" s="11"/>
-      <c r="CM71" s="11"/>
-      <c r="CN71" s="11"/>
-      <c r="CO71" s="11"/>
-      <c r="CP71" s="11"/>
-      <c r="CQ71" s="11"/>
-      <c r="CR71" s="11"/>
-      <c r="CS71" s="11"/>
-      <c r="CT71" s="11"/>
-      <c r="CU71" s="11"/>
-      <c r="CV71" s="11"/>
-      <c r="CW71" s="11"/>
-      <c r="CX71" s="11"/>
-      <c r="CY71" s="11"/>
-      <c r="CZ71" s="11"/>
-      <c r="DA71" s="11"/>
-      <c r="DB71" s="11"/>
-      <c r="DC71" s="11"/>
-      <c r="DD71" s="11"/>
-      <c r="DE71" s="11"/>
-      <c r="DF71" s="11"/>
-      <c r="DG71" s="11"/>
-      <c r="DH71" s="11"/>
-      <c r="DI71" s="11"/>
-      <c r="DJ71" s="11"/>
-      <c r="DK71" s="11"/>
-      <c r="DL71" s="11"/>
-      <c r="DM71" s="11"/>
-      <c r="DN71" s="11"/>
-      <c r="DO71" s="11"/>
-      <c r="DP71" s="11"/>
-      <c r="DQ71" s="11"/>
-      <c r="DR71" s="11"/>
-      <c r="DS71" s="11"/>
-      <c r="DT71" s="11"/>
-      <c r="DU71" s="11"/>
-      <c r="DV71" s="11"/>
-      <c r="DW71" s="11"/>
-      <c r="DX71" s="11"/>
-      <c r="DY71" s="11"/>
-      <c r="DZ71" s="11"/>
-      <c r="EA71" s="11"/>
-      <c r="EB71" s="11"/>
-      <c r="EC71" s="11"/>
-      <c r="ED71" s="11"/>
-      <c r="EE71" s="11"/>
-      <c r="EF71" s="11"/>
-      <c r="EG71" s="11"/>
-      <c r="EH71" s="11"/>
-      <c r="EI71" s="11"/>
-      <c r="EJ71" s="11"/>
-      <c r="EK71" s="11"/>
-      <c r="EL71" s="11"/>
-      <c r="EM71" s="11"/>
-      <c r="EN71" s="11"/>
-      <c r="EO71" s="11"/>
-      <c r="EP71" s="11"/>
-      <c r="EQ71" s="11"/>
-      <c r="ER71" s="11"/>
-      <c r="ES71" s="11"/>
-      <c r="ET71" s="11"/>
-      <c r="EU71" s="11"/>
-      <c r="EV71" s="11"/>
-      <c r="EW71" s="11"/>
-      <c r="EX71" s="11"/>
-      <c r="EY71" s="11"/>
-      <c r="EZ71" s="11"/>
-      <c r="FA71" s="11"/>
-      <c r="FB71" s="11"/>
-      <c r="FC71" s="11"/>
-      <c r="FD71" s="11"/>
-      <c r="FE71" s="11"/>
-      <c r="FF71" s="11"/>
-      <c r="FG71" s="11"/>
-      <c r="FH71" s="11"/>
-      <c r="FI71" s="11"/>
-      <c r="FJ71" s="11"/>
-      <c r="FK71" s="11"/>
-      <c r="FL71" s="11"/>
-      <c r="FM71" s="11"/>
-      <c r="FN71" s="11"/>
-      <c r="FO71" s="11"/>
-      <c r="FP71" s="11"/>
-      <c r="FQ71" s="11"/>
-      <c r="FR71" s="11"/>
-      <c r="FS71" s="11"/>
-      <c r="FT71" s="11"/>
-      <c r="FU71" s="11"/>
-      <c r="FV71" s="11"/>
-      <c r="FW71" s="11"/>
-      <c r="FX71" s="11"/>
-      <c r="FY71" s="11"/>
-      <c r="FZ71" s="11"/>
-      <c r="GA71" s="11"/>
-      <c r="GB71" s="11"/>
-      <c r="GC71" s="11"/>
-      <c r="GD71" s="11"/>
-      <c r="GE71" s="11"/>
-      <c r="GF71" s="11"/>
-      <c r="GG71" s="11"/>
-      <c r="GH71" s="11"/>
-      <c r="GI71" s="11"/>
-      <c r="GJ71" s="11"/>
-      <c r="GK71" s="11"/>
-      <c r="GL71" s="11"/>
-      <c r="GM71" s="11"/>
-      <c r="GN71" s="11"/>
-      <c r="GO71" s="11"/>
-      <c r="GP71" s="11"/>
-      <c r="GQ71" s="11"/>
-      <c r="GR71" s="11"/>
-      <c r="GS71" s="11"/>
-      <c r="GT71" s="11"/>
-      <c r="GU71" s="11"/>
-      <c r="GV71" s="11"/>
-      <c r="GW71" s="11"/>
-      <c r="GX71" s="11"/>
-      <c r="GY71" s="11"/>
-      <c r="GZ71" s="11"/>
-      <c r="HA71" s="11"/>
-      <c r="HB71" s="11"/>
-      <c r="HC71" s="11"/>
-      <c r="HD71" s="11"/>
-      <c r="HE71" s="11"/>
-      <c r="HF71" s="11"/>
-      <c r="HG71" s="11"/>
-      <c r="HH71" s="11"/>
-      <c r="HI71" s="11"/>
-      <c r="HJ71" s="11"/>
-      <c r="HK71" s="11"/>
-      <c r="HL71" s="11"/>
-      <c r="HM71" s="11"/>
-      <c r="HN71" s="11"/>
-      <c r="HO71" s="11"/>
-      <c r="HP71" s="11"/>
-      <c r="HQ71" s="11"/>
-      <c r="HR71" s="11"/>
-      <c r="HS71" s="11"/>
-      <c r="HT71" s="11"/>
-      <c r="HU71" s="11"/>
-      <c r="HV71" s="11"/>
-      <c r="HW71" s="11"/>
-      <c r="HX71" s="11"/>
-      <c r="HY71" s="11"/>
-      <c r="HZ71" s="11"/>
-      <c r="IA71" s="11"/>
-      <c r="IB71" s="11"/>
-      <c r="IC71" s="11"/>
-      <c r="ID71" s="11"/>
-      <c r="IE71" s="11"/>
-      <c r="IF71" s="11"/>
-      <c r="IG71" s="11"/>
-      <c r="IH71" s="11"/>
-      <c r="II71" s="11"/>
-      <c r="IJ71" s="11"/>
-      <c r="IK71" s="11"/>
-      <c r="IL71" s="11"/>
-      <c r="IM71" s="11"/>
-      <c r="IN71" s="11"/>
-      <c r="IO71" s="11"/>
-      <c r="IP71" s="11"/>
-      <c r="IQ71" s="11"/>
-      <c r="IR71" s="11"/>
-      <c r="IS71" s="11"/>
-      <c r="IT71" s="11"/>
-      <c r="IU71" s="11"/>
-      <c r="IV71" s="11"/>
-      <c r="IW71" s="11"/>
-      <c r="IX71" s="11"/>
-      <c r="IY71" s="11"/>
-      <c r="IZ71" s="11"/>
-      <c r="JA71" s="11"/>
-      <c r="JB71" s="11"/>
-      <c r="JC71" s="11"/>
-      <c r="JD71" s="11"/>
-      <c r="JE71" s="11"/>
-      <c r="JF71" s="11"/>
-      <c r="JG71" s="11"/>
-      <c r="JH71" s="11"/>
-      <c r="JI71" s="11"/>
-      <c r="JJ71" s="11"/>
-      <c r="JK71" s="11"/>
-      <c r="JL71" s="11"/>
-      <c r="JM71" s="11"/>
-      <c r="JN71" s="11"/>
-      <c r="JO71" s="11"/>
-      <c r="JP71" s="11"/>
-      <c r="JQ71" s="11"/>
-      <c r="JR71" s="11"/>
-      <c r="JS71" s="11"/>
-      <c r="JT71" s="11"/>
-      <c r="JU71" s="11"/>
-      <c r="JV71" s="11"/>
-      <c r="JW71" s="11"/>
-      <c r="JX71" s="11"/>
-      <c r="JY71" s="11"/>
-      <c r="JZ71" s="11"/>
-      <c r="KA71" s="11"/>
-      <c r="KB71" s="11"/>
-      <c r="KC71" s="11"/>
-      <c r="KD71" s="11"/>
-      <c r="KE71" s="11"/>
-      <c r="KF71" s="11"/>
-      <c r="KG71" s="11"/>
-      <c r="KH71" s="11"/>
-      <c r="KI71" s="11"/>
-      <c r="KJ71" s="11"/>
-      <c r="KK71" s="11"/>
-      <c r="KL71" s="11"/>
-      <c r="KM71" s="11"/>
-      <c r="KN71" s="11"/>
-      <c r="KO71" s="11"/>
-      <c r="KP71" s="11"/>
-      <c r="KQ71" s="11"/>
-      <c r="KR71" s="11"/>
-      <c r="KS71" s="11"/>
-      <c r="KT71" s="11"/>
-      <c r="KU71" s="11"/>
-      <c r="KV71" s="11"/>
-      <c r="KW71" s="11"/>
-      <c r="KX71" s="11"/>
-      <c r="KY71" s="11"/>
-      <c r="KZ71" s="11"/>
-      <c r="LA71" s="11"/>
-      <c r="LB71" s="11"/>
-      <c r="LC71" s="11"/>
-      <c r="LD71" s="11"/>
-      <c r="LE71" s="11"/>
-      <c r="LF71" s="11"/>
-      <c r="LG71" s="11"/>
-      <c r="LH71" s="11"/>
-      <c r="LI71" s="11"/>
-      <c r="LJ71" s="11"/>
-      <c r="LK71" s="11"/>
-      <c r="LL71" s="11"/>
-      <c r="LM71" s="11"/>
-      <c r="LN71" s="11"/>
-      <c r="LO71" s="11"/>
-      <c r="LP71" s="11"/>
-      <c r="LQ71" s="11"/>
-      <c r="LR71" s="11"/>
-      <c r="LS71" s="11"/>
-      <c r="LT71" s="11"/>
-      <c r="LU71" s="11"/>
-      <c r="LV71" s="11"/>
-      <c r="LW71" s="11"/>
-      <c r="LX71" s="11"/>
-      <c r="LY71" s="11"/>
-      <c r="LZ71" s="11"/>
-      <c r="MA71" s="11"/>
-      <c r="MB71" s="11"/>
-      <c r="MC71" s="11"/>
-      <c r="MD71" s="11"/>
-      <c r="ME71" s="11"/>
-      <c r="MF71" s="11"/>
-      <c r="MG71" s="11"/>
-      <c r="MH71" s="11"/>
-      <c r="MI71" s="11"/>
-      <c r="MJ71" s="11"/>
-      <c r="MK71" s="11"/>
-      <c r="ML71" s="11"/>
-      <c r="MM71" s="11"/>
-      <c r="MN71" s="11"/>
-      <c r="MO71" s="11"/>
-      <c r="MP71" s="11"/>
-      <c r="MQ71" s="11"/>
-      <c r="MR71" s="11"/>
-      <c r="MS71" s="11"/>
-      <c r="MT71" s="11"/>
-      <c r="MU71" s="11"/>
-      <c r="MV71" s="11"/>
-      <c r="MW71" s="11"/>
-      <c r="MX71" s="11"/>
-      <c r="MY71" s="11"/>
-      <c r="MZ71" s="11"/>
-      <c r="NA71" s="11"/>
-      <c r="NB71" s="11"/>
-      <c r="NC71" s="11"/>
-      <c r="ND71" s="11"/>
-      <c r="NE71" s="11"/>
-      <c r="NF71" s="11"/>
-      <c r="NG71" s="11"/>
-      <c r="NH71" s="11"/>
-      <c r="NI71" s="11"/>
-      <c r="NJ71" s="11"/>
-      <c r="NK71" s="11"/>
-      <c r="NL71" s="11"/>
-      <c r="NM71" s="11"/>
-      <c r="NN71" s="11"/>
-      <c r="NO71" s="11"/>
-      <c r="NP71" s="11"/>
-      <c r="NQ71" s="11"/>
-      <c r="NR71" s="11"/>
-      <c r="NS71" s="11"/>
-      <c r="NT71" s="11"/>
-      <c r="NU71" s="11"/>
-      <c r="NV71" s="11"/>
-      <c r="NW71" s="11"/>
-      <c r="NX71" s="11"/>
-      <c r="NY71" s="11"/>
-      <c r="NZ71" s="11"/>
-      <c r="OA71" s="11"/>
-      <c r="OB71" s="11"/>
-      <c r="OC71" s="11"/>
-      <c r="OD71" s="11"/>
-      <c r="OE71" s="11"/>
-      <c r="OF71" s="11"/>
-      <c r="OG71" s="11"/>
-      <c r="OH71" s="11"/>
-      <c r="OI71" s="11"/>
-      <c r="OJ71" s="11"/>
-      <c r="OK71" s="11"/>
-      <c r="OL71" s="11"/>
-      <c r="OM71" s="11"/>
-      <c r="ON71" s="11"/>
-      <c r="OO71" s="11"/>
-      <c r="OP71" s="11"/>
-      <c r="OQ71" s="11"/>
-      <c r="OR71" s="11"/>
-      <c r="OS71" s="11"/>
-      <c r="OT71" s="11"/>
-      <c r="OU71" s="11"/>
-      <c r="OV71" s="11"/>
-      <c r="OW71" s="11"/>
-      <c r="OX71" s="11"/>
-      <c r="OY71" s="11"/>
-      <c r="OZ71" s="11"/>
-      <c r="PA71" s="11"/>
-      <c r="PB71" s="11"/>
-      <c r="PC71" s="11"/>
-      <c r="PD71" s="11"/>
-      <c r="PE71" s="11"/>
-      <c r="PF71" s="11"/>
-      <c r="PG71" s="11"/>
-      <c r="PH71" s="11"/>
-      <c r="PI71" s="11"/>
-      <c r="PJ71" s="11"/>
-      <c r="PK71" s="11"/>
-      <c r="PL71" s="11"/>
-      <c r="PM71" s="11"/>
-      <c r="PN71" s="11"/>
-      <c r="PO71" s="11"/>
-      <c r="PP71" s="11"/>
-      <c r="PQ71" s="11"/>
-      <c r="PR71" s="11"/>
-      <c r="PS71" s="11"/>
-      <c r="PT71" s="11"/>
-      <c r="PU71" s="11"/>
-      <c r="PV71" s="11"/>
-      <c r="PW71" s="11"/>
-      <c r="PX71" s="11"/>
-      <c r="PY71" s="11"/>
-      <c r="PZ71" s="11"/>
-      <c r="QA71" s="11"/>
-      <c r="QB71" s="11"/>
-      <c r="QC71" s="11"/>
-      <c r="QD71" s="11"/>
-      <c r="QE71" s="11"/>
-      <c r="QF71" s="11"/>
-      <c r="QG71" s="11"/>
-      <c r="QH71" s="11"/>
-      <c r="QI71" s="11"/>
-      <c r="QJ71" s="11"/>
-      <c r="QK71" s="11"/>
-      <c r="QL71" s="11"/>
-      <c r="QM71" s="11"/>
-      <c r="QN71" s="11"/>
-      <c r="QO71" s="11"/>
-      <c r="QP71" s="11"/>
-      <c r="QQ71" s="11"/>
-      <c r="QR71" s="11"/>
-      <c r="QS71" s="11"/>
-      <c r="QT71" s="11"/>
-      <c r="QU71" s="11"/>
-      <c r="QV71" s="11"/>
-      <c r="QW71" s="11"/>
-      <c r="QX71" s="11"/>
-      <c r="QY71" s="11"/>
-      <c r="QZ71" s="11"/>
-      <c r="RA71" s="11"/>
-      <c r="RB71" s="11"/>
-      <c r="RC71" s="11"/>
-      <c r="RD71" s="11"/>
-      <c r="RE71" s="11"/>
-      <c r="RF71" s="11"/>
-      <c r="RG71" s="11"/>
-      <c r="RH71" s="11"/>
-      <c r="RI71" s="11"/>
-      <c r="RJ71" s="11"/>
-      <c r="RK71" s="11"/>
-      <c r="RL71" s="11"/>
-      <c r="RM71" s="11"/>
-      <c r="RN71" s="11"/>
-      <c r="RO71" s="11"/>
-      <c r="RP71" s="11"/>
-      <c r="RQ71" s="11"/>
-      <c r="RR71" s="11"/>
-      <c r="RS71" s="11"/>
-      <c r="RT71" s="11"/>
-      <c r="RU71" s="11"/>
-      <c r="RV71" s="11"/>
-      <c r="RW71" s="11"/>
-      <c r="RX71" s="11"/>
-      <c r="RY71" s="11"/>
-      <c r="RZ71" s="11"/>
-      <c r="SA71" s="11"/>
-      <c r="SB71" s="11"/>
-      <c r="SC71" s="11"/>
-      <c r="SD71" s="11"/>
-      <c r="SE71" s="11"/>
-      <c r="SF71" s="11"/>
-      <c r="SG71" s="11"/>
-      <c r="SH71" s="11"/>
-      <c r="SI71" s="11"/>
-      <c r="SJ71" s="11"/>
-      <c r="SK71" s="11"/>
-      <c r="SL71" s="11"/>
-      <c r="SM71" s="11"/>
-      <c r="SN71" s="11"/>
-      <c r="SO71" s="11"/>
-      <c r="SP71" s="11"/>
-      <c r="SQ71" s="11"/>
-      <c r="SR71" s="11"/>
-      <c r="SS71" s="11"/>
-      <c r="ST71" s="11"/>
-      <c r="SU71" s="11"/>
-      <c r="SV71" s="11"/>
-      <c r="SW71" s="11"/>
-      <c r="SX71" s="11"/>
-      <c r="SY71" s="11"/>
-      <c r="SZ71" s="11"/>
-      <c r="TA71" s="11"/>
-      <c r="TB71" s="11"/>
-      <c r="TC71" s="11"/>
-      <c r="TD71" s="11"/>
-      <c r="TE71" s="11"/>
-      <c r="TF71" s="11"/>
-      <c r="TG71" s="11"/>
-      <c r="TH71" s="11"/>
-      <c r="TI71" s="11"/>
-      <c r="TJ71" s="11"/>
-      <c r="TK71" s="11"/>
-      <c r="TL71" s="11"/>
-      <c r="TM71" s="11"/>
-      <c r="TN71" s="11"/>
-      <c r="TO71" s="11"/>
-      <c r="TP71" s="11"/>
-      <c r="TQ71" s="11"/>
-      <c r="TR71" s="11"/>
-      <c r="TS71" s="11"/>
-      <c r="TT71" s="11"/>
-      <c r="TU71" s="11"/>
-      <c r="TV71" s="11"/>
-      <c r="TW71" s="11"/>
-      <c r="TX71" s="11"/>
-      <c r="TY71" s="11"/>
-      <c r="TZ71" s="11"/>
-      <c r="UA71" s="11"/>
-      <c r="UB71" s="11"/>
-      <c r="UC71" s="11"/>
-      <c r="UD71" s="11"/>
-      <c r="UE71" s="11"/>
-      <c r="UF71" s="11"/>
-      <c r="UG71" s="11"/>
-      <c r="UH71" s="11"/>
-      <c r="UI71" s="11"/>
-      <c r="UJ71" s="11"/>
-      <c r="UK71" s="11"/>
-      <c r="UL71" s="11"/>
-      <c r="UM71" s="11"/>
-      <c r="UN71" s="11"/>
-      <c r="UO71" s="11"/>
-      <c r="UP71" s="11"/>
-      <c r="UQ71" s="11"/>
-      <c r="UR71" s="11"/>
-      <c r="US71" s="11"/>
-      <c r="UT71" s="11"/>
-      <c r="UU71" s="11"/>
-      <c r="UV71" s="11"/>
-      <c r="UW71" s="11"/>
-      <c r="UX71" s="11"/>
-      <c r="UY71" s="11"/>
-      <c r="UZ71" s="11"/>
-      <c r="VA71" s="11"/>
-      <c r="VB71" s="11"/>
-      <c r="VC71" s="11"/>
-      <c r="VD71" s="11"/>
-      <c r="VE71" s="11"/>
-      <c r="VF71" s="11"/>
-      <c r="VG71" s="11"/>
-      <c r="VH71" s="11"/>
-      <c r="VI71" s="11"/>
-      <c r="VJ71" s="11"/>
-      <c r="VK71" s="11"/>
-      <c r="VL71" s="11"/>
-      <c r="VM71" s="11"/>
-      <c r="VN71" s="11"/>
-      <c r="VO71" s="11"/>
-      <c r="VP71" s="11"/>
-      <c r="VQ71" s="11"/>
-      <c r="VR71" s="11"/>
-      <c r="VS71" s="11"/>
-      <c r="VT71" s="11"/>
-      <c r="VU71" s="11"/>
-      <c r="VV71" s="11"/>
-      <c r="VW71" s="11"/>
-      <c r="VX71" s="11"/>
-      <c r="VY71" s="11"/>
-      <c r="VZ71" s="11"/>
-      <c r="WA71" s="11"/>
-      <c r="WB71" s="11"/>
-      <c r="WC71" s="11"/>
-      <c r="WD71" s="11"/>
-      <c r="WE71" s="11"/>
-      <c r="WF71" s="11"/>
-      <c r="WG71" s="11"/>
-      <c r="WH71" s="11"/>
-      <c r="WI71" s="11"/>
-      <c r="WJ71" s="11"/>
-      <c r="WK71" s="11"/>
-      <c r="WL71" s="11"/>
-      <c r="WM71" s="11"/>
-      <c r="WN71" s="11"/>
-      <c r="WO71" s="11"/>
-      <c r="WP71" s="11"/>
-      <c r="WQ71" s="11"/>
-      <c r="WR71" s="11"/>
-      <c r="WS71" s="11"/>
-      <c r="WT71" s="11"/>
-      <c r="WU71" s="11"/>
-      <c r="WV71" s="11"/>
-      <c r="WW71" s="11"/>
-      <c r="WX71" s="11"/>
-      <c r="WY71" s="11"/>
-      <c r="WZ71" s="11"/>
-      <c r="XA71" s="11"/>
-      <c r="XB71" s="11"/>
-      <c r="XC71" s="11"/>
-      <c r="XD71" s="11"/>
-      <c r="XE71" s="11"/>
-      <c r="XF71" s="11"/>
-      <c r="XG71" s="11"/>
-      <c r="XH71" s="11"/>
-      <c r="XI71" s="11"/>
-      <c r="XJ71" s="11"/>
-      <c r="XK71" s="11"/>
-      <c r="XL71" s="11"/>
-      <c r="XM71" s="11"/>
-      <c r="XN71" s="11"/>
-      <c r="XO71" s="11"/>
-      <c r="XP71" s="11"/>
-      <c r="XQ71" s="11"/>
-      <c r="XR71" s="11"/>
-      <c r="XS71" s="11"/>
-      <c r="XT71" s="11"/>
-      <c r="XU71" s="11"/>
-      <c r="XV71" s="11"/>
-      <c r="XW71" s="11"/>
-      <c r="XX71" s="11"/>
-      <c r="XY71" s="11"/>
-      <c r="XZ71" s="11"/>
-      <c r="YA71" s="11"/>
-      <c r="YB71" s="11"/>
-      <c r="YC71" s="11"/>
-      <c r="YD71" s="11"/>
-      <c r="YE71" s="11"/>
-      <c r="YF71" s="11"/>
-      <c r="YG71" s="11"/>
-      <c r="YH71" s="11"/>
-      <c r="YI71" s="11"/>
-      <c r="YJ71" s="11"/>
-      <c r="YK71" s="11"/>
-      <c r="YL71" s="11"/>
-      <c r="YM71" s="11"/>
-      <c r="YN71" s="11"/>
-      <c r="YO71" s="11"/>
-      <c r="YP71" s="11"/>
-      <c r="YQ71" s="11"/>
-      <c r="YR71" s="11"/>
-      <c r="YS71" s="11"/>
-      <c r="YT71" s="11"/>
-      <c r="YU71" s="11"/>
-      <c r="YV71" s="11"/>
-      <c r="YW71" s="11"/>
-      <c r="YX71" s="11"/>
-      <c r="YY71" s="11"/>
-      <c r="YZ71" s="11"/>
-      <c r="ZA71" s="11"/>
-      <c r="ZB71" s="11"/>
-      <c r="ZC71" s="11"/>
-      <c r="ZD71" s="11"/>
-      <c r="ZE71" s="11"/>
-      <c r="ZF71" s="11"/>
-      <c r="ZG71" s="11"/>
-      <c r="ZH71" s="11"/>
-      <c r="ZI71" s="11"/>
-      <c r="ZJ71" s="11"/>
-      <c r="ZK71" s="11"/>
-      <c r="ZL71" s="11"/>
-      <c r="ZM71" s="11"/>
-      <c r="ZN71" s="11"/>
-      <c r="ZO71" s="11"/>
-      <c r="ZP71" s="11"/>
-      <c r="ZQ71" s="11"/>
-      <c r="ZR71" s="11"/>
-      <c r="ZS71" s="11"/>
-      <c r="ZT71" s="11"/>
-      <c r="ZU71" s="11"/>
-      <c r="ZV71" s="11"/>
-      <c r="ZW71" s="11"/>
-      <c r="ZX71" s="11"/>
-      <c r="ZY71" s="11"/>
-      <c r="ZZ71" s="11"/>
-      <c r="AAA71" s="11"/>
-      <c r="AAB71" s="11"/>
-      <c r="AAC71" s="11"/>
-      <c r="AAD71" s="11"/>
-      <c r="AAE71" s="11"/>
-      <c r="AAF71" s="11"/>
-      <c r="AAG71" s="11"/>
-      <c r="AAH71" s="11"/>
-      <c r="AAI71" s="11"/>
-      <c r="AAJ71" s="11"/>
-      <c r="AAK71" s="11"/>
-      <c r="AAL71" s="11"/>
-      <c r="AAM71" s="11"/>
-      <c r="AAN71" s="11"/>
-      <c r="AAO71" s="11"/>
-      <c r="AAP71" s="11"/>
-      <c r="AAQ71" s="11"/>
-      <c r="AAR71" s="11"/>
-      <c r="AAS71" s="11"/>
-      <c r="AAT71" s="11"/>
-      <c r="AAU71" s="11"/>
-      <c r="AAV71" s="11"/>
-      <c r="AAW71" s="11"/>
-      <c r="AAX71" s="11"/>
-      <c r="AAY71" s="11"/>
-      <c r="AAZ71" s="11"/>
-      <c r="ABA71" s="11"/>
-      <c r="ABB71" s="11"/>
-      <c r="ABC71" s="11"/>
-      <c r="ABD71" s="11"/>
-      <c r="ABE71" s="11"/>
-      <c r="ABF71" s="11"/>
-      <c r="ABG71" s="11"/>
-      <c r="ABH71" s="11"/>
-      <c r="ABI71" s="11"/>
-      <c r="ABJ71" s="11"/>
-      <c r="ABK71" s="11"/>
-      <c r="ABL71" s="11"/>
-      <c r="ABM71" s="11"/>
-      <c r="ABN71" s="11"/>
-      <c r="ABO71" s="11"/>
-      <c r="ABP71" s="11"/>
-      <c r="ABQ71" s="11"/>
-      <c r="ABR71" s="11"/>
-      <c r="ABS71" s="11"/>
-      <c r="ABT71" s="11"/>
-      <c r="ABU71" s="11"/>
-      <c r="ABV71" s="11"/>
-      <c r="ABW71" s="11"/>
-      <c r="ABX71" s="11"/>
-      <c r="ABY71" s="11"/>
-      <c r="ABZ71" s="11"/>
-      <c r="ACA71" s="11"/>
-      <c r="ACB71" s="11"/>
-      <c r="ACC71" s="11"/>
-      <c r="ACD71" s="11"/>
-      <c r="ACE71" s="11"/>
-      <c r="ACF71" s="11"/>
-      <c r="ACG71" s="11"/>
-      <c r="ACH71" s="11"/>
-      <c r="ACI71" s="11"/>
-      <c r="ACJ71" s="11"/>
-      <c r="ACK71" s="11"/>
-      <c r="ACL71" s="11"/>
-      <c r="ACM71" s="11"/>
-      <c r="ACN71" s="11"/>
-      <c r="ACO71" s="11"/>
-      <c r="ACP71" s="11"/>
-      <c r="ACQ71" s="11"/>
-      <c r="ACR71" s="11"/>
-      <c r="ACS71" s="11"/>
-      <c r="ACT71" s="11"/>
-      <c r="ACU71" s="11"/>
-      <c r="ACV71" s="11"/>
-      <c r="ACW71" s="11"/>
-      <c r="ACX71" s="11"/>
-      <c r="ACY71" s="11"/>
-      <c r="ACZ71" s="11"/>
-      <c r="ADA71" s="11"/>
-      <c r="ADB71" s="11"/>
-      <c r="ADC71" s="11"/>
-      <c r="ADD71" s="11"/>
-      <c r="ADE71" s="11"/>
-      <c r="ADF71" s="11"/>
-      <c r="ADG71" s="11"/>
-      <c r="ADH71" s="11"/>
-      <c r="ADI71" s="11"/>
-      <c r="ADJ71" s="11"/>
-      <c r="ADK71" s="11"/>
-      <c r="ADL71" s="11"/>
-      <c r="ADM71" s="11"/>
-      <c r="ADN71" s="11"/>
-      <c r="ADO71" s="11"/>
-      <c r="ADP71" s="11"/>
-      <c r="ADQ71" s="11"/>
-      <c r="ADR71" s="11"/>
-      <c r="ADS71" s="11"/>
-      <c r="ADT71" s="11"/>
-      <c r="ADU71" s="11"/>
-      <c r="ADV71" s="11"/>
-      <c r="ADW71" s="11"/>
-      <c r="ADX71" s="11"/>
-      <c r="ADY71" s="11"/>
-      <c r="ADZ71" s="11"/>
-      <c r="AEA71" s="11"/>
-      <c r="AEB71" s="11"/>
-      <c r="AEC71" s="11"/>
-      <c r="AED71" s="11"/>
-      <c r="AEE71" s="11"/>
-      <c r="AEF71" s="11"/>
-      <c r="AEG71" s="11"/>
-      <c r="AEH71" s="11"/>
-      <c r="AEI71" s="11"/>
-      <c r="AEJ71" s="11"/>
-      <c r="AEK71" s="11"/>
-      <c r="AEL71" s="11"/>
-      <c r="AEM71" s="11"/>
-      <c r="AEN71" s="11"/>
-      <c r="AEO71" s="11"/>
-      <c r="AEP71" s="11"/>
-      <c r="AEQ71" s="11"/>
-      <c r="AER71" s="11"/>
-      <c r="AES71" s="11"/>
-      <c r="AET71" s="11"/>
-      <c r="AEU71" s="11"/>
-      <c r="AEV71" s="11"/>
-      <c r="AEW71" s="11"/>
-      <c r="AEX71" s="11"/>
-      <c r="AEY71" s="11"/>
-      <c r="AEZ71" s="11"/>
-      <c r="AFA71" s="11"/>
-      <c r="AFB71" s="11"/>
-      <c r="AFC71" s="11"/>
-      <c r="AFD71" s="11"/>
-      <c r="AFE71" s="11"/>
-      <c r="AFF71" s="11"/>
-      <c r="AFG71" s="11"/>
-      <c r="AFH71" s="11"/>
-      <c r="AFI71" s="11"/>
-      <c r="AFJ71" s="11"/>
-      <c r="AFK71" s="11"/>
-      <c r="AFL71" s="11"/>
-      <c r="AFM71" s="11"/>
-      <c r="AFN71" s="11"/>
-      <c r="AFO71" s="11"/>
-      <c r="AFP71" s="11"/>
-      <c r="AFQ71" s="11"/>
-      <c r="AFR71" s="11"/>
-      <c r="AFS71" s="11"/>
-      <c r="AFT71" s="11"/>
-      <c r="AFU71" s="11"/>
-      <c r="AFV71" s="11"/>
-      <c r="AFW71" s="11"/>
-      <c r="AFX71" s="11"/>
-      <c r="AFY71" s="11"/>
-      <c r="AFZ71" s="11"/>
-      <c r="AGA71" s="11"/>
-      <c r="AGB71" s="11"/>
-      <c r="AGC71" s="11"/>
-      <c r="AGD71" s="11"/>
-      <c r="AGE71" s="11"/>
-      <c r="AGF71" s="11"/>
-      <c r="AGG71" s="11"/>
-      <c r="AGH71" s="11"/>
-      <c r="AGI71" s="11"/>
-      <c r="AGJ71" s="11"/>
-      <c r="AGK71" s="11"/>
-      <c r="AGL71" s="11"/>
-      <c r="AGM71" s="11"/>
-      <c r="AGN71" s="11"/>
-      <c r="AGO71" s="11"/>
-      <c r="AGP71" s="11"/>
-      <c r="AGQ71" s="11"/>
-      <c r="AGR71" s="11"/>
-      <c r="AGS71" s="11"/>
-      <c r="AGT71" s="11"/>
-      <c r="AGU71" s="11"/>
-      <c r="AGV71" s="11"/>
-      <c r="AGW71" s="11"/>
-      <c r="AGX71" s="11"/>
-      <c r="AGY71" s="11"/>
-      <c r="AGZ71" s="11"/>
-      <c r="AHA71" s="11"/>
-      <c r="AHB71" s="11"/>
-      <c r="AHC71" s="11"/>
-      <c r="AHD71" s="11"/>
-      <c r="AHE71" s="11"/>
-      <c r="AHF71" s="11"/>
-      <c r="AHG71" s="11"/>
-      <c r="AHH71" s="11"/>
-      <c r="AHI71" s="11"/>
-      <c r="AHJ71" s="11"/>
-      <c r="AHK71" s="11"/>
-      <c r="AHL71" s="11"/>
-      <c r="AHM71" s="11"/>
-      <c r="AHN71" s="11"/>
-      <c r="AHO71" s="11"/>
-      <c r="AHP71" s="11"/>
-      <c r="AHQ71" s="11"/>
-      <c r="AHR71" s="11"/>
-      <c r="AHS71" s="11"/>
-      <c r="AHT71" s="11"/>
-      <c r="AHU71" s="11"/>
-      <c r="AHV71" s="11"/>
-      <c r="AHW71" s="11"/>
-      <c r="AHX71" s="11"/>
-      <c r="AHY71" s="11"/>
-      <c r="AHZ71" s="11"/>
-      <c r="AIA71" s="11"/>
-      <c r="AIB71" s="11"/>
-      <c r="AIC71" s="11"/>
-      <c r="AID71" s="11"/>
-      <c r="AIE71" s="11"/>
-      <c r="AIF71" s="11"/>
-      <c r="AIG71" s="11"/>
-      <c r="AIH71" s="11"/>
-      <c r="AII71" s="11"/>
-      <c r="AIJ71" s="11"/>
-      <c r="AIK71" s="11"/>
-      <c r="AIL71" s="11"/>
-      <c r="AIM71" s="11"/>
-      <c r="AIN71" s="11"/>
-      <c r="AIO71" s="11"/>
-      <c r="AIP71" s="11"/>
-      <c r="AIQ71" s="11"/>
-      <c r="AIR71" s="11"/>
-      <c r="AIS71" s="11"/>
-      <c r="AIT71" s="11"/>
-      <c r="AIU71" s="11"/>
-      <c r="AIV71" s="11"/>
-      <c r="AIW71" s="11"/>
-      <c r="AIX71" s="11"/>
-      <c r="AIY71" s="11"/>
-      <c r="AIZ71" s="11"/>
-      <c r="AJA71" s="11"/>
-      <c r="AJB71" s="11"/>
-      <c r="AJC71" s="11"/>
-      <c r="AJD71" s="11"/>
-      <c r="AJE71" s="11"/>
-      <c r="AJF71" s="11"/>
-      <c r="AJG71" s="11"/>
-      <c r="AJH71" s="11"/>
-      <c r="AJI71" s="11"/>
-      <c r="AJJ71" s="11"/>
-      <c r="AJK71" s="11"/>
-      <c r="AJL71" s="11"/>
-      <c r="AJM71" s="11"/>
-      <c r="AJN71" s="11"/>
-      <c r="AJO71" s="11"/>
-      <c r="AJP71" s="11"/>
-      <c r="AJQ71" s="11"/>
-      <c r="AJR71" s="11"/>
-      <c r="AJS71" s="11"/>
-      <c r="AJT71" s="11"/>
-      <c r="AJU71" s="11"/>
-      <c r="AJV71" s="11"/>
-      <c r="AJW71" s="11"/>
-      <c r="AJX71" s="11"/>
-      <c r="AJY71" s="11"/>
-      <c r="AJZ71" s="11"/>
-      <c r="AKA71" s="11"/>
-      <c r="AKB71" s="11"/>
-      <c r="AKC71" s="11"/>
-      <c r="AKD71" s="11"/>
-      <c r="AKE71" s="11"/>
-      <c r="AKF71" s="11"/>
-      <c r="AKG71" s="11"/>
-      <c r="AKH71" s="11"/>
-      <c r="AKI71" s="11"/>
-      <c r="AKJ71" s="11"/>
-      <c r="AKK71" s="11"/>
-      <c r="AKL71" s="11"/>
-      <c r="AKM71" s="11"/>
-      <c r="AKN71" s="11"/>
-      <c r="AKO71" s="11"/>
-      <c r="AKP71" s="11"/>
-      <c r="AKQ71" s="11"/>
-      <c r="AKR71" s="11"/>
-      <c r="AKS71" s="11"/>
-      <c r="AKT71" s="11"/>
-      <c r="AKU71" s="11"/>
-      <c r="AKV71" s="11"/>
-      <c r="AKW71" s="11"/>
-      <c r="AKX71" s="11"/>
-      <c r="AKY71" s="11"/>
-      <c r="AKZ71" s="11"/>
-      <c r="ALA71" s="11"/>
-      <c r="ALB71" s="11"/>
-      <c r="ALC71" s="11"/>
-      <c r="ALD71" s="11"/>
-      <c r="ALE71" s="11"/>
-      <c r="ALF71" s="11"/>
-      <c r="ALG71" s="11"/>
-      <c r="ALH71" s="11"/>
-      <c r="ALI71" s="11"/>
-      <c r="ALJ71" s="11"/>
-      <c r="ALK71" s="11"/>
-      <c r="ALL71" s="11"/>
-      <c r="ALM71" s="11"/>
-      <c r="ALN71" s="11"/>
-      <c r="ALO71" s="11"/>
-      <c r="ALP71" s="11"/>
-      <c r="ALQ71" s="11"/>
-      <c r="ALR71" s="11"/>
-      <c r="ALS71" s="11"/>
-      <c r="ALT71" s="11"/>
-      <c r="ALU71" s="11"/>
-      <c r="ALV71" s="11"/>
-      <c r="ALW71" s="11"/>
-      <c r="ALX71" s="11"/>
-      <c r="ALY71" s="11"/>
-      <c r="ALZ71" s="11"/>
-      <c r="AMA71" s="11"/>
-      <c r="AMB71" s="11"/>
-      <c r="AMC71" s="11"/>
-      <c r="AMD71" s="11"/>
-      <c r="AME71" s="11"/>
-      <c r="AMF71" s="11"/>
-      <c r="AMG71" s="11"/>
-      <c r="AMH71" s="11"/>
-      <c r="AMI71" s="11"/>
-      <c r="AMJ71" s="11"/>
-    </row>
-    <row r="1048415" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048416" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048417" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="71" s="11" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="72" s="11" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="73" s="11" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="74" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="11"/>
+      <c r="B74" s="11"/>
+      <c r="C74" s="11"/>
+      <c r="D74" s="11"/>
+      <c r="E74" s="11"/>
+      <c r="F74" s="11"/>
+      <c r="G74" s="11"/>
+      <c r="H74" s="11"/>
+      <c r="I74" s="11"/>
+      <c r="J74" s="11"/>
+      <c r="K74" s="11"/>
+      <c r="L74" s="11"/>
+      <c r="M74" s="11"/>
+      <c r="N74" s="11"/>
+      <c r="O74" s="11"/>
+      <c r="P74" s="11"/>
+      <c r="Q74" s="11"/>
+      <c r="R74" s="11"/>
+      <c r="S74" s="11"/>
+      <c r="T74" s="11"/>
+      <c r="U74" s="11"/>
+      <c r="V74" s="11"/>
+      <c r="W74" s="11"/>
+      <c r="X74" s="11"/>
+      <c r="Y74" s="11"/>
+      <c r="Z74" s="11"/>
+      <c r="AA74" s="11"/>
+      <c r="AB74" s="11"/>
+      <c r="AC74" s="11"/>
+      <c r="AD74" s="11"/>
+      <c r="AE74" s="11"/>
+      <c r="AF74" s="11"/>
+      <c r="AG74" s="11"/>
+      <c r="AH74" s="11"/>
+      <c r="AI74" s="11"/>
+      <c r="AJ74" s="11"/>
+      <c r="AK74" s="11"/>
+      <c r="AL74" s="11"/>
+      <c r="AM74" s="11"/>
+      <c r="AN74" s="11"/>
+      <c r="AO74" s="11"/>
+      <c r="AP74" s="11"/>
+      <c r="AQ74" s="11"/>
+      <c r="AR74" s="11"/>
+      <c r="AS74" s="11"/>
+      <c r="AT74" s="11"/>
+      <c r="AU74" s="11"/>
+      <c r="AV74" s="11"/>
+      <c r="AW74" s="11"/>
+      <c r="AX74" s="11"/>
+      <c r="AY74" s="11"/>
+      <c r="AZ74" s="11"/>
+      <c r="BA74" s="11"/>
+      <c r="BB74" s="11"/>
+      <c r="BC74" s="11"/>
+      <c r="BD74" s="11"/>
+      <c r="BE74" s="11"/>
+      <c r="BF74" s="11"/>
+      <c r="BG74" s="11"/>
+      <c r="BH74" s="11"/>
+      <c r="BI74" s="11"/>
+      <c r="BJ74" s="11"/>
+      <c r="BK74" s="11"/>
+      <c r="BL74" s="11"/>
+      <c r="BM74" s="11"/>
+      <c r="BN74" s="11"/>
+      <c r="BO74" s="11"/>
+      <c r="BP74" s="11"/>
+      <c r="BQ74" s="11"/>
+      <c r="BR74" s="11"/>
+      <c r="BS74" s="11"/>
+      <c r="BT74" s="11"/>
+      <c r="BU74" s="11"/>
+      <c r="BV74" s="11"/>
+      <c r="BW74" s="11"/>
+      <c r="BX74" s="11"/>
+      <c r="BY74" s="11"/>
+      <c r="BZ74" s="11"/>
+      <c r="CA74" s="11"/>
+      <c r="CB74" s="11"/>
+      <c r="CC74" s="11"/>
+      <c r="CD74" s="11"/>
+      <c r="CE74" s="11"/>
+      <c r="CF74" s="11"/>
+      <c r="CG74" s="11"/>
+      <c r="CH74" s="11"/>
+      <c r="CI74" s="11"/>
+      <c r="CJ74" s="11"/>
+      <c r="CK74" s="11"/>
+      <c r="CL74" s="11"/>
+      <c r="CM74" s="11"/>
+      <c r="CN74" s="11"/>
+      <c r="CO74" s="11"/>
+      <c r="CP74" s="11"/>
+      <c r="CQ74" s="11"/>
+      <c r="CR74" s="11"/>
+      <c r="CS74" s="11"/>
+      <c r="CT74" s="11"/>
+      <c r="CU74" s="11"/>
+      <c r="CV74" s="11"/>
+      <c r="CW74" s="11"/>
+      <c r="CX74" s="11"/>
+      <c r="CY74" s="11"/>
+      <c r="CZ74" s="11"/>
+      <c r="DA74" s="11"/>
+      <c r="DB74" s="11"/>
+      <c r="DC74" s="11"/>
+      <c r="DD74" s="11"/>
+      <c r="DE74" s="11"/>
+      <c r="DF74" s="11"/>
+      <c r="DG74" s="11"/>
+      <c r="DH74" s="11"/>
+      <c r="DI74" s="11"/>
+      <c r="DJ74" s="11"/>
+      <c r="DK74" s="11"/>
+      <c r="DL74" s="11"/>
+      <c r="DM74" s="11"/>
+      <c r="DN74" s="11"/>
+      <c r="DO74" s="11"/>
+      <c r="DP74" s="11"/>
+      <c r="DQ74" s="11"/>
+      <c r="DR74" s="11"/>
+      <c r="DS74" s="11"/>
+      <c r="DT74" s="11"/>
+      <c r="DU74" s="11"/>
+      <c r="DV74" s="11"/>
+      <c r="DW74" s="11"/>
+      <c r="DX74" s="11"/>
+      <c r="DY74" s="11"/>
+      <c r="DZ74" s="11"/>
+      <c r="EA74" s="11"/>
+      <c r="EB74" s="11"/>
+      <c r="EC74" s="11"/>
+      <c r="ED74" s="11"/>
+      <c r="EE74" s="11"/>
+      <c r="EF74" s="11"/>
+      <c r="EG74" s="11"/>
+      <c r="EH74" s="11"/>
+      <c r="EI74" s="11"/>
+      <c r="EJ74" s="11"/>
+      <c r="EK74" s="11"/>
+      <c r="EL74" s="11"/>
+      <c r="EM74" s="11"/>
+      <c r="EN74" s="11"/>
+      <c r="EO74" s="11"/>
+      <c r="EP74" s="11"/>
+      <c r="EQ74" s="11"/>
+      <c r="ER74" s="11"/>
+      <c r="ES74" s="11"/>
+      <c r="ET74" s="11"/>
+      <c r="EU74" s="11"/>
+      <c r="EV74" s="11"/>
+      <c r="EW74" s="11"/>
+      <c r="EX74" s="11"/>
+      <c r="EY74" s="11"/>
+      <c r="EZ74" s="11"/>
+      <c r="FA74" s="11"/>
+      <c r="FB74" s="11"/>
+      <c r="FC74" s="11"/>
+      <c r="FD74" s="11"/>
+      <c r="FE74" s="11"/>
+      <c r="FF74" s="11"/>
+      <c r="FG74" s="11"/>
+      <c r="FH74" s="11"/>
+      <c r="FI74" s="11"/>
+      <c r="FJ74" s="11"/>
+      <c r="FK74" s="11"/>
+      <c r="FL74" s="11"/>
+      <c r="FM74" s="11"/>
+      <c r="FN74" s="11"/>
+      <c r="FO74" s="11"/>
+      <c r="FP74" s="11"/>
+      <c r="FQ74" s="11"/>
+      <c r="FR74" s="11"/>
+      <c r="FS74" s="11"/>
+      <c r="FT74" s="11"/>
+      <c r="FU74" s="11"/>
+      <c r="FV74" s="11"/>
+      <c r="FW74" s="11"/>
+      <c r="FX74" s="11"/>
+      <c r="FY74" s="11"/>
+      <c r="FZ74" s="11"/>
+      <c r="GA74" s="11"/>
+      <c r="GB74" s="11"/>
+      <c r="GC74" s="11"/>
+      <c r="GD74" s="11"/>
+      <c r="GE74" s="11"/>
+      <c r="GF74" s="11"/>
+      <c r="GG74" s="11"/>
+      <c r="GH74" s="11"/>
+      <c r="GI74" s="11"/>
+      <c r="GJ74" s="11"/>
+      <c r="GK74" s="11"/>
+      <c r="GL74" s="11"/>
+      <c r="GM74" s="11"/>
+      <c r="GN74" s="11"/>
+      <c r="GO74" s="11"/>
+      <c r="GP74" s="11"/>
+      <c r="GQ74" s="11"/>
+      <c r="GR74" s="11"/>
+      <c r="GS74" s="11"/>
+      <c r="GT74" s="11"/>
+      <c r="GU74" s="11"/>
+      <c r="GV74" s="11"/>
+      <c r="GW74" s="11"/>
+      <c r="GX74" s="11"/>
+      <c r="GY74" s="11"/>
+      <c r="GZ74" s="11"/>
+      <c r="HA74" s="11"/>
+      <c r="HB74" s="11"/>
+      <c r="HC74" s="11"/>
+      <c r="HD74" s="11"/>
+      <c r="HE74" s="11"/>
+      <c r="HF74" s="11"/>
+      <c r="HG74" s="11"/>
+      <c r="HH74" s="11"/>
+      <c r="HI74" s="11"/>
+      <c r="HJ74" s="11"/>
+      <c r="HK74" s="11"/>
+      <c r="HL74" s="11"/>
+      <c r="HM74" s="11"/>
+      <c r="HN74" s="11"/>
+      <c r="HO74" s="11"/>
+      <c r="HP74" s="11"/>
+      <c r="HQ74" s="11"/>
+      <c r="HR74" s="11"/>
+      <c r="HS74" s="11"/>
+      <c r="HT74" s="11"/>
+      <c r="HU74" s="11"/>
+      <c r="HV74" s="11"/>
+      <c r="HW74" s="11"/>
+      <c r="HX74" s="11"/>
+      <c r="HY74" s="11"/>
+      <c r="HZ74" s="11"/>
+      <c r="IA74" s="11"/>
+      <c r="IB74" s="11"/>
+      <c r="IC74" s="11"/>
+      <c r="ID74" s="11"/>
+      <c r="IE74" s="11"/>
+      <c r="IF74" s="11"/>
+      <c r="IG74" s="11"/>
+      <c r="IH74" s="11"/>
+      <c r="II74" s="11"/>
+      <c r="IJ74" s="11"/>
+      <c r="IK74" s="11"/>
+      <c r="IL74" s="11"/>
+      <c r="IM74" s="11"/>
+      <c r="IN74" s="11"/>
+      <c r="IO74" s="11"/>
+      <c r="IP74" s="11"/>
+      <c r="IQ74" s="11"/>
+      <c r="IR74" s="11"/>
+      <c r="IS74" s="11"/>
+      <c r="IT74" s="11"/>
+      <c r="IU74" s="11"/>
+      <c r="IV74" s="11"/>
+      <c r="IW74" s="11"/>
+      <c r="IX74" s="11"/>
+      <c r="IY74" s="11"/>
+      <c r="IZ74" s="11"/>
+      <c r="JA74" s="11"/>
+      <c r="JB74" s="11"/>
+      <c r="JC74" s="11"/>
+      <c r="JD74" s="11"/>
+      <c r="JE74" s="11"/>
+      <c r="JF74" s="11"/>
+      <c r="JG74" s="11"/>
+      <c r="JH74" s="11"/>
+      <c r="JI74" s="11"/>
+      <c r="JJ74" s="11"/>
+      <c r="JK74" s="11"/>
+      <c r="JL74" s="11"/>
+      <c r="JM74" s="11"/>
+      <c r="JN74" s="11"/>
+      <c r="JO74" s="11"/>
+      <c r="JP74" s="11"/>
+      <c r="JQ74" s="11"/>
+      <c r="JR74" s="11"/>
+      <c r="JS74" s="11"/>
+      <c r="JT74" s="11"/>
+      <c r="JU74" s="11"/>
+      <c r="JV74" s="11"/>
+      <c r="JW74" s="11"/>
+      <c r="JX74" s="11"/>
+      <c r="JY74" s="11"/>
+      <c r="JZ74" s="11"/>
+      <c r="KA74" s="11"/>
+      <c r="KB74" s="11"/>
+      <c r="KC74" s="11"/>
+      <c r="KD74" s="11"/>
+      <c r="KE74" s="11"/>
+      <c r="KF74" s="11"/>
+      <c r="KG74" s="11"/>
+      <c r="KH74" s="11"/>
+      <c r="KI74" s="11"/>
+      <c r="KJ74" s="11"/>
+      <c r="KK74" s="11"/>
+      <c r="KL74" s="11"/>
+      <c r="KM74" s="11"/>
+      <c r="KN74" s="11"/>
+      <c r="KO74" s="11"/>
+      <c r="KP74" s="11"/>
+      <c r="KQ74" s="11"/>
+      <c r="KR74" s="11"/>
+      <c r="KS74" s="11"/>
+      <c r="KT74" s="11"/>
+      <c r="KU74" s="11"/>
+      <c r="KV74" s="11"/>
+      <c r="KW74" s="11"/>
+      <c r="KX74" s="11"/>
+      <c r="KY74" s="11"/>
+      <c r="KZ74" s="11"/>
+      <c r="LA74" s="11"/>
+      <c r="LB74" s="11"/>
+      <c r="LC74" s="11"/>
+      <c r="LD74" s="11"/>
+      <c r="LE74" s="11"/>
+      <c r="LF74" s="11"/>
+      <c r="LG74" s="11"/>
+      <c r="LH74" s="11"/>
+      <c r="LI74" s="11"/>
+      <c r="LJ74" s="11"/>
+      <c r="LK74" s="11"/>
+      <c r="LL74" s="11"/>
+      <c r="LM74" s="11"/>
+      <c r="LN74" s="11"/>
+      <c r="LO74" s="11"/>
+      <c r="LP74" s="11"/>
+      <c r="LQ74" s="11"/>
+      <c r="LR74" s="11"/>
+      <c r="LS74" s="11"/>
+      <c r="LT74" s="11"/>
+      <c r="LU74" s="11"/>
+      <c r="LV74" s="11"/>
+      <c r="LW74" s="11"/>
+      <c r="LX74" s="11"/>
+      <c r="LY74" s="11"/>
+      <c r="LZ74" s="11"/>
+      <c r="MA74" s="11"/>
+      <c r="MB74" s="11"/>
+      <c r="MC74" s="11"/>
+      <c r="MD74" s="11"/>
+      <c r="ME74" s="11"/>
+      <c r="MF74" s="11"/>
+      <c r="MG74" s="11"/>
+      <c r="MH74" s="11"/>
+      <c r="MI74" s="11"/>
+      <c r="MJ74" s="11"/>
+      <c r="MK74" s="11"/>
+      <c r="ML74" s="11"/>
+      <c r="MM74" s="11"/>
+      <c r="MN74" s="11"/>
+      <c r="MO74" s="11"/>
+      <c r="MP74" s="11"/>
+      <c r="MQ74" s="11"/>
+      <c r="MR74" s="11"/>
+      <c r="MS74" s="11"/>
+      <c r="MT74" s="11"/>
+      <c r="MU74" s="11"/>
+      <c r="MV74" s="11"/>
+      <c r="MW74" s="11"/>
+      <c r="MX74" s="11"/>
+      <c r="MY74" s="11"/>
+      <c r="MZ74" s="11"/>
+      <c r="NA74" s="11"/>
+      <c r="NB74" s="11"/>
+      <c r="NC74" s="11"/>
+      <c r="ND74" s="11"/>
+      <c r="NE74" s="11"/>
+      <c r="NF74" s="11"/>
+      <c r="NG74" s="11"/>
+      <c r="NH74" s="11"/>
+      <c r="NI74" s="11"/>
+      <c r="NJ74" s="11"/>
+      <c r="NK74" s="11"/>
+      <c r="NL74" s="11"/>
+      <c r="NM74" s="11"/>
+      <c r="NN74" s="11"/>
+      <c r="NO74" s="11"/>
+      <c r="NP74" s="11"/>
+      <c r="NQ74" s="11"/>
+      <c r="NR74" s="11"/>
+      <c r="NS74" s="11"/>
+      <c r="NT74" s="11"/>
+      <c r="NU74" s="11"/>
+      <c r="NV74" s="11"/>
+      <c r="NW74" s="11"/>
+      <c r="NX74" s="11"/>
+      <c r="NY74" s="11"/>
+      <c r="NZ74" s="11"/>
+      <c r="OA74" s="11"/>
+      <c r="OB74" s="11"/>
+      <c r="OC74" s="11"/>
+      <c r="OD74" s="11"/>
+      <c r="OE74" s="11"/>
+      <c r="OF74" s="11"/>
+      <c r="OG74" s="11"/>
+      <c r="OH74" s="11"/>
+      <c r="OI74" s="11"/>
+      <c r="OJ74" s="11"/>
+      <c r="OK74" s="11"/>
+      <c r="OL74" s="11"/>
+      <c r="OM74" s="11"/>
+      <c r="ON74" s="11"/>
+      <c r="OO74" s="11"/>
+      <c r="OP74" s="11"/>
+      <c r="OQ74" s="11"/>
+      <c r="OR74" s="11"/>
+      <c r="OS74" s="11"/>
+      <c r="OT74" s="11"/>
+      <c r="OU74" s="11"/>
+      <c r="OV74" s="11"/>
+      <c r="OW74" s="11"/>
+      <c r="OX74" s="11"/>
+      <c r="OY74" s="11"/>
+      <c r="OZ74" s="11"/>
+      <c r="PA74" s="11"/>
+      <c r="PB74" s="11"/>
+      <c r="PC74" s="11"/>
+      <c r="PD74" s="11"/>
+      <c r="PE74" s="11"/>
+      <c r="PF74" s="11"/>
+      <c r="PG74" s="11"/>
+      <c r="PH74" s="11"/>
+      <c r="PI74" s="11"/>
+      <c r="PJ74" s="11"/>
+      <c r="PK74" s="11"/>
+      <c r="PL74" s="11"/>
+      <c r="PM74" s="11"/>
+      <c r="PN74" s="11"/>
+      <c r="PO74" s="11"/>
+      <c r="PP74" s="11"/>
+      <c r="PQ74" s="11"/>
+      <c r="PR74" s="11"/>
+      <c r="PS74" s="11"/>
+      <c r="PT74" s="11"/>
+      <c r="PU74" s="11"/>
+      <c r="PV74" s="11"/>
+      <c r="PW74" s="11"/>
+      <c r="PX74" s="11"/>
+      <c r="PY74" s="11"/>
+      <c r="PZ74" s="11"/>
+      <c r="QA74" s="11"/>
+      <c r="QB74" s="11"/>
+      <c r="QC74" s="11"/>
+      <c r="QD74" s="11"/>
+      <c r="QE74" s="11"/>
+      <c r="QF74" s="11"/>
+      <c r="QG74" s="11"/>
+      <c r="QH74" s="11"/>
+      <c r="QI74" s="11"/>
+      <c r="QJ74" s="11"/>
+      <c r="QK74" s="11"/>
+      <c r="QL74" s="11"/>
+      <c r="QM74" s="11"/>
+      <c r="QN74" s="11"/>
+      <c r="QO74" s="11"/>
+      <c r="QP74" s="11"/>
+      <c r="QQ74" s="11"/>
+      <c r="QR74" s="11"/>
+      <c r="QS74" s="11"/>
+      <c r="QT74" s="11"/>
+      <c r="QU74" s="11"/>
+      <c r="QV74" s="11"/>
+      <c r="QW74" s="11"/>
+      <c r="QX74" s="11"/>
+      <c r="QY74" s="11"/>
+      <c r="QZ74" s="11"/>
+      <c r="RA74" s="11"/>
+      <c r="RB74" s="11"/>
+      <c r="RC74" s="11"/>
+      <c r="RD74" s="11"/>
+      <c r="RE74" s="11"/>
+      <c r="RF74" s="11"/>
+      <c r="RG74" s="11"/>
+      <c r="RH74" s="11"/>
+      <c r="RI74" s="11"/>
+      <c r="RJ74" s="11"/>
+      <c r="RK74" s="11"/>
+      <c r="RL74" s="11"/>
+      <c r="RM74" s="11"/>
+      <c r="RN74" s="11"/>
+      <c r="RO74" s="11"/>
+      <c r="RP74" s="11"/>
+      <c r="RQ74" s="11"/>
+      <c r="RR74" s="11"/>
+      <c r="RS74" s="11"/>
+      <c r="RT74" s="11"/>
+      <c r="RU74" s="11"/>
+      <c r="RV74" s="11"/>
+      <c r="RW74" s="11"/>
+      <c r="RX74" s="11"/>
+      <c r="RY74" s="11"/>
+      <c r="RZ74" s="11"/>
+      <c r="SA74" s="11"/>
+      <c r="SB74" s="11"/>
+      <c r="SC74" s="11"/>
+      <c r="SD74" s="11"/>
+      <c r="SE74" s="11"/>
+      <c r="SF74" s="11"/>
+      <c r="SG74" s="11"/>
+      <c r="SH74" s="11"/>
+      <c r="SI74" s="11"/>
+      <c r="SJ74" s="11"/>
+      <c r="SK74" s="11"/>
+      <c r="SL74" s="11"/>
+      <c r="SM74" s="11"/>
+      <c r="SN74" s="11"/>
+      <c r="SO74" s="11"/>
+      <c r="SP74" s="11"/>
+      <c r="SQ74" s="11"/>
+      <c r="SR74" s="11"/>
+      <c r="SS74" s="11"/>
+      <c r="ST74" s="11"/>
+      <c r="SU74" s="11"/>
+      <c r="SV74" s="11"/>
+      <c r="SW74" s="11"/>
+      <c r="SX74" s="11"/>
+      <c r="SY74" s="11"/>
+      <c r="SZ74" s="11"/>
+      <c r="TA74" s="11"/>
+      <c r="TB74" s="11"/>
+      <c r="TC74" s="11"/>
+      <c r="TD74" s="11"/>
+      <c r="TE74" s="11"/>
+      <c r="TF74" s="11"/>
+      <c r="TG74" s="11"/>
+      <c r="TH74" s="11"/>
+      <c r="TI74" s="11"/>
+      <c r="TJ74" s="11"/>
+      <c r="TK74" s="11"/>
+      <c r="TL74" s="11"/>
+      <c r="TM74" s="11"/>
+      <c r="TN74" s="11"/>
+      <c r="TO74" s="11"/>
+      <c r="TP74" s="11"/>
+      <c r="TQ74" s="11"/>
+      <c r="TR74" s="11"/>
+      <c r="TS74" s="11"/>
+      <c r="TT74" s="11"/>
+      <c r="TU74" s="11"/>
+      <c r="TV74" s="11"/>
+      <c r="TW74" s="11"/>
+      <c r="TX74" s="11"/>
+      <c r="TY74" s="11"/>
+      <c r="TZ74" s="11"/>
+      <c r="UA74" s="11"/>
+      <c r="UB74" s="11"/>
+      <c r="UC74" s="11"/>
+      <c r="UD74" s="11"/>
+      <c r="UE74" s="11"/>
+      <c r="UF74" s="11"/>
+      <c r="UG74" s="11"/>
+      <c r="UH74" s="11"/>
+      <c r="UI74" s="11"/>
+      <c r="UJ74" s="11"/>
+      <c r="UK74" s="11"/>
+      <c r="UL74" s="11"/>
+      <c r="UM74" s="11"/>
+      <c r="UN74" s="11"/>
+      <c r="UO74" s="11"/>
+      <c r="UP74" s="11"/>
+      <c r="UQ74" s="11"/>
+      <c r="UR74" s="11"/>
+      <c r="US74" s="11"/>
+      <c r="UT74" s="11"/>
+      <c r="UU74" s="11"/>
+      <c r="UV74" s="11"/>
+      <c r="UW74" s="11"/>
+      <c r="UX74" s="11"/>
+      <c r="UY74" s="11"/>
+      <c r="UZ74" s="11"/>
+      <c r="VA74" s="11"/>
+      <c r="VB74" s="11"/>
+      <c r="VC74" s="11"/>
+      <c r="VD74" s="11"/>
+      <c r="VE74" s="11"/>
+      <c r="VF74" s="11"/>
+      <c r="VG74" s="11"/>
+      <c r="VH74" s="11"/>
+      <c r="VI74" s="11"/>
+      <c r="VJ74" s="11"/>
+      <c r="VK74" s="11"/>
+      <c r="VL74" s="11"/>
+      <c r="VM74" s="11"/>
+      <c r="VN74" s="11"/>
+      <c r="VO74" s="11"/>
+      <c r="VP74" s="11"/>
+      <c r="VQ74" s="11"/>
+      <c r="VR74" s="11"/>
+      <c r="VS74" s="11"/>
+      <c r="VT74" s="11"/>
+      <c r="VU74" s="11"/>
+      <c r="VV74" s="11"/>
+      <c r="VW74" s="11"/>
+      <c r="VX74" s="11"/>
+      <c r="VY74" s="11"/>
+      <c r="VZ74" s="11"/>
+      <c r="WA74" s="11"/>
+      <c r="WB74" s="11"/>
+      <c r="WC74" s="11"/>
+      <c r="WD74" s="11"/>
+      <c r="WE74" s="11"/>
+      <c r="WF74" s="11"/>
+      <c r="WG74" s="11"/>
+      <c r="WH74" s="11"/>
+      <c r="WI74" s="11"/>
+      <c r="WJ74" s="11"/>
+      <c r="WK74" s="11"/>
+      <c r="WL74" s="11"/>
+      <c r="WM74" s="11"/>
+      <c r="WN74" s="11"/>
+      <c r="WO74" s="11"/>
+      <c r="WP74" s="11"/>
+      <c r="WQ74" s="11"/>
+      <c r="WR74" s="11"/>
+      <c r="WS74" s="11"/>
+      <c r="WT74" s="11"/>
+      <c r="WU74" s="11"/>
+      <c r="WV74" s="11"/>
+      <c r="WW74" s="11"/>
+      <c r="WX74" s="11"/>
+      <c r="WY74" s="11"/>
+      <c r="WZ74" s="11"/>
+      <c r="XA74" s="11"/>
+      <c r="XB74" s="11"/>
+      <c r="XC74" s="11"/>
+      <c r="XD74" s="11"/>
+      <c r="XE74" s="11"/>
+      <c r="XF74" s="11"/>
+      <c r="XG74" s="11"/>
+      <c r="XH74" s="11"/>
+      <c r="XI74" s="11"/>
+      <c r="XJ74" s="11"/>
+      <c r="XK74" s="11"/>
+      <c r="XL74" s="11"/>
+      <c r="XM74" s="11"/>
+      <c r="XN74" s="11"/>
+      <c r="XO74" s="11"/>
+      <c r="XP74" s="11"/>
+      <c r="XQ74" s="11"/>
+      <c r="XR74" s="11"/>
+      <c r="XS74" s="11"/>
+      <c r="XT74" s="11"/>
+      <c r="XU74" s="11"/>
+      <c r="XV74" s="11"/>
+      <c r="XW74" s="11"/>
+      <c r="XX74" s="11"/>
+      <c r="XY74" s="11"/>
+      <c r="XZ74" s="11"/>
+      <c r="YA74" s="11"/>
+      <c r="YB74" s="11"/>
+      <c r="YC74" s="11"/>
+      <c r="YD74" s="11"/>
+      <c r="YE74" s="11"/>
+      <c r="YF74" s="11"/>
+      <c r="YG74" s="11"/>
+      <c r="YH74" s="11"/>
+      <c r="YI74" s="11"/>
+      <c r="YJ74" s="11"/>
+      <c r="YK74" s="11"/>
+      <c r="YL74" s="11"/>
+      <c r="YM74" s="11"/>
+      <c r="YN74" s="11"/>
+      <c r="YO74" s="11"/>
+      <c r="YP74" s="11"/>
+      <c r="YQ74" s="11"/>
+      <c r="YR74" s="11"/>
+      <c r="YS74" s="11"/>
+      <c r="YT74" s="11"/>
+      <c r="YU74" s="11"/>
+      <c r="YV74" s="11"/>
+      <c r="YW74" s="11"/>
+      <c r="YX74" s="11"/>
+      <c r="YY74" s="11"/>
+      <c r="YZ74" s="11"/>
+      <c r="ZA74" s="11"/>
+      <c r="ZB74" s="11"/>
+      <c r="ZC74" s="11"/>
+      <c r="ZD74" s="11"/>
+      <c r="ZE74" s="11"/>
+      <c r="ZF74" s="11"/>
+      <c r="ZG74" s="11"/>
+      <c r="ZH74" s="11"/>
+      <c r="ZI74" s="11"/>
+      <c r="ZJ74" s="11"/>
+      <c r="ZK74" s="11"/>
+      <c r="ZL74" s="11"/>
+      <c r="ZM74" s="11"/>
+      <c r="ZN74" s="11"/>
+      <c r="ZO74" s="11"/>
+      <c r="ZP74" s="11"/>
+      <c r="ZQ74" s="11"/>
+      <c r="ZR74" s="11"/>
+      <c r="ZS74" s="11"/>
+      <c r="ZT74" s="11"/>
+      <c r="ZU74" s="11"/>
+      <c r="ZV74" s="11"/>
+      <c r="ZW74" s="11"/>
+      <c r="ZX74" s="11"/>
+      <c r="ZY74" s="11"/>
+      <c r="ZZ74" s="11"/>
+      <c r="AAA74" s="11"/>
+      <c r="AAB74" s="11"/>
+      <c r="AAC74" s="11"/>
+      <c r="AAD74" s="11"/>
+      <c r="AAE74" s="11"/>
+      <c r="AAF74" s="11"/>
+      <c r="AAG74" s="11"/>
+      <c r="AAH74" s="11"/>
+      <c r="AAI74" s="11"/>
+      <c r="AAJ74" s="11"/>
+      <c r="AAK74" s="11"/>
+      <c r="AAL74" s="11"/>
+      <c r="AAM74" s="11"/>
+      <c r="AAN74" s="11"/>
+      <c r="AAO74" s="11"/>
+      <c r="AAP74" s="11"/>
+      <c r="AAQ74" s="11"/>
+      <c r="AAR74" s="11"/>
+      <c r="AAS74" s="11"/>
+      <c r="AAT74" s="11"/>
+      <c r="AAU74" s="11"/>
+      <c r="AAV74" s="11"/>
+      <c r="AAW74" s="11"/>
+      <c r="AAX74" s="11"/>
+      <c r="AAY74" s="11"/>
+      <c r="AAZ74" s="11"/>
+      <c r="ABA74" s="11"/>
+      <c r="ABB74" s="11"/>
+      <c r="ABC74" s="11"/>
+      <c r="ABD74" s="11"/>
+      <c r="ABE74" s="11"/>
+      <c r="ABF74" s="11"/>
+      <c r="ABG74" s="11"/>
+      <c r="ABH74" s="11"/>
+      <c r="ABI74" s="11"/>
+      <c r="ABJ74" s="11"/>
+      <c r="ABK74" s="11"/>
+      <c r="ABL74" s="11"/>
+      <c r="ABM74" s="11"/>
+      <c r="ABN74" s="11"/>
+      <c r="ABO74" s="11"/>
+      <c r="ABP74" s="11"/>
+      <c r="ABQ74" s="11"/>
+      <c r="ABR74" s="11"/>
+      <c r="ABS74" s="11"/>
+      <c r="ABT74" s="11"/>
+      <c r="ABU74" s="11"/>
+      <c r="ABV74" s="11"/>
+      <c r="ABW74" s="11"/>
+      <c r="ABX74" s="11"/>
+      <c r="ABY74" s="11"/>
+      <c r="ABZ74" s="11"/>
+      <c r="ACA74" s="11"/>
+      <c r="ACB74" s="11"/>
+      <c r="ACC74" s="11"/>
+      <c r="ACD74" s="11"/>
+      <c r="ACE74" s="11"/>
+      <c r="ACF74" s="11"/>
+      <c r="ACG74" s="11"/>
+      <c r="ACH74" s="11"/>
+      <c r="ACI74" s="11"/>
+      <c r="ACJ74" s="11"/>
+      <c r="ACK74" s="11"/>
+      <c r="ACL74" s="11"/>
+      <c r="ACM74" s="11"/>
+      <c r="ACN74" s="11"/>
+      <c r="ACO74" s="11"/>
+      <c r="ACP74" s="11"/>
+      <c r="ACQ74" s="11"/>
+      <c r="ACR74" s="11"/>
+      <c r="ACS74" s="11"/>
+      <c r="ACT74" s="11"/>
+      <c r="ACU74" s="11"/>
+      <c r="ACV74" s="11"/>
+      <c r="ACW74" s="11"/>
+      <c r="ACX74" s="11"/>
+      <c r="ACY74" s="11"/>
+      <c r="ACZ74" s="11"/>
+      <c r="ADA74" s="11"/>
+      <c r="ADB74" s="11"/>
+      <c r="ADC74" s="11"/>
+      <c r="ADD74" s="11"/>
+      <c r="ADE74" s="11"/>
+      <c r="ADF74" s="11"/>
+      <c r="ADG74" s="11"/>
+      <c r="ADH74" s="11"/>
+      <c r="ADI74" s="11"/>
+      <c r="ADJ74" s="11"/>
+      <c r="ADK74" s="11"/>
+      <c r="ADL74" s="11"/>
+      <c r="ADM74" s="11"/>
+      <c r="ADN74" s="11"/>
+      <c r="ADO74" s="11"/>
+      <c r="ADP74" s="11"/>
+      <c r="ADQ74" s="11"/>
+      <c r="ADR74" s="11"/>
+      <c r="ADS74" s="11"/>
+      <c r="ADT74" s="11"/>
+      <c r="ADU74" s="11"/>
+      <c r="ADV74" s="11"/>
+      <c r="ADW74" s="11"/>
+      <c r="ADX74" s="11"/>
+      <c r="ADY74" s="11"/>
+      <c r="ADZ74" s="11"/>
+      <c r="AEA74" s="11"/>
+      <c r="AEB74" s="11"/>
+      <c r="AEC74" s="11"/>
+      <c r="AED74" s="11"/>
+      <c r="AEE74" s="11"/>
+      <c r="AEF74" s="11"/>
+      <c r="AEG74" s="11"/>
+      <c r="AEH74" s="11"/>
+      <c r="AEI74" s="11"/>
+      <c r="AEJ74" s="11"/>
+      <c r="AEK74" s="11"/>
+      <c r="AEL74" s="11"/>
+      <c r="AEM74" s="11"/>
+      <c r="AEN74" s="11"/>
+      <c r="AEO74" s="11"/>
+      <c r="AEP74" s="11"/>
+      <c r="AEQ74" s="11"/>
+      <c r="AER74" s="11"/>
+      <c r="AES74" s="11"/>
+      <c r="AET74" s="11"/>
+      <c r="AEU74" s="11"/>
+      <c r="AEV74" s="11"/>
+      <c r="AEW74" s="11"/>
+      <c r="AEX74" s="11"/>
+      <c r="AEY74" s="11"/>
+      <c r="AEZ74" s="11"/>
+      <c r="AFA74" s="11"/>
+      <c r="AFB74" s="11"/>
+      <c r="AFC74" s="11"/>
+      <c r="AFD74" s="11"/>
+      <c r="AFE74" s="11"/>
+      <c r="AFF74" s="11"/>
+      <c r="AFG74" s="11"/>
+      <c r="AFH74" s="11"/>
+      <c r="AFI74" s="11"/>
+      <c r="AFJ74" s="11"/>
+      <c r="AFK74" s="11"/>
+      <c r="AFL74" s="11"/>
+      <c r="AFM74" s="11"/>
+      <c r="AFN74" s="11"/>
+      <c r="AFO74" s="11"/>
+      <c r="AFP74" s="11"/>
+      <c r="AFQ74" s="11"/>
+      <c r="AFR74" s="11"/>
+      <c r="AFS74" s="11"/>
+      <c r="AFT74" s="11"/>
+      <c r="AFU74" s="11"/>
+      <c r="AFV74" s="11"/>
+      <c r="AFW74" s="11"/>
+      <c r="AFX74" s="11"/>
+      <c r="AFY74" s="11"/>
+      <c r="AFZ74" s="11"/>
+      <c r="AGA74" s="11"/>
+      <c r="AGB74" s="11"/>
+      <c r="AGC74" s="11"/>
+      <c r="AGD74" s="11"/>
+      <c r="AGE74" s="11"/>
+      <c r="AGF74" s="11"/>
+      <c r="AGG74" s="11"/>
+      <c r="AGH74" s="11"/>
+      <c r="AGI74" s="11"/>
+      <c r="AGJ74" s="11"/>
+      <c r="AGK74" s="11"/>
+      <c r="AGL74" s="11"/>
+      <c r="AGM74" s="11"/>
+      <c r="AGN74" s="11"/>
+      <c r="AGO74" s="11"/>
+      <c r="AGP74" s="11"/>
+      <c r="AGQ74" s="11"/>
+      <c r="AGR74" s="11"/>
+      <c r="AGS74" s="11"/>
+      <c r="AGT74" s="11"/>
+      <c r="AGU74" s="11"/>
+      <c r="AGV74" s="11"/>
+      <c r="AGW74" s="11"/>
+      <c r="AGX74" s="11"/>
+      <c r="AGY74" s="11"/>
+      <c r="AGZ74" s="11"/>
+      <c r="AHA74" s="11"/>
+      <c r="AHB74" s="11"/>
+      <c r="AHC74" s="11"/>
+      <c r="AHD74" s="11"/>
+      <c r="AHE74" s="11"/>
+      <c r="AHF74" s="11"/>
+      <c r="AHG74" s="11"/>
+      <c r="AHH74" s="11"/>
+      <c r="AHI74" s="11"/>
+      <c r="AHJ74" s="11"/>
+      <c r="AHK74" s="11"/>
+      <c r="AHL74" s="11"/>
+      <c r="AHM74" s="11"/>
+      <c r="AHN74" s="11"/>
+      <c r="AHO74" s="11"/>
+      <c r="AHP74" s="11"/>
+      <c r="AHQ74" s="11"/>
+      <c r="AHR74" s="11"/>
+      <c r="AHS74" s="11"/>
+      <c r="AHT74" s="11"/>
+      <c r="AHU74" s="11"/>
+      <c r="AHV74" s="11"/>
+      <c r="AHW74" s="11"/>
+      <c r="AHX74" s="11"/>
+      <c r="AHY74" s="11"/>
+      <c r="AHZ74" s="11"/>
+      <c r="AIA74" s="11"/>
+      <c r="AIB74" s="11"/>
+      <c r="AIC74" s="11"/>
+      <c r="AID74" s="11"/>
+      <c r="AIE74" s="11"/>
+      <c r="AIF74" s="11"/>
+      <c r="AIG74" s="11"/>
+      <c r="AIH74" s="11"/>
+      <c r="AII74" s="11"/>
+      <c r="AIJ74" s="11"/>
+      <c r="AIK74" s="11"/>
+      <c r="AIL74" s="11"/>
+      <c r="AIM74" s="11"/>
+      <c r="AIN74" s="11"/>
+      <c r="AIO74" s="11"/>
+      <c r="AIP74" s="11"/>
+      <c r="AIQ74" s="11"/>
+      <c r="AIR74" s="11"/>
+      <c r="AIS74" s="11"/>
+      <c r="AIT74" s="11"/>
+      <c r="AIU74" s="11"/>
+      <c r="AIV74" s="11"/>
+      <c r="AIW74" s="11"/>
+      <c r="AIX74" s="11"/>
+      <c r="AIY74" s="11"/>
+      <c r="AIZ74" s="11"/>
+      <c r="AJA74" s="11"/>
+      <c r="AJB74" s="11"/>
+      <c r="AJC74" s="11"/>
+      <c r="AJD74" s="11"/>
+      <c r="AJE74" s="11"/>
+      <c r="AJF74" s="11"/>
+      <c r="AJG74" s="11"/>
+      <c r="AJH74" s="11"/>
+      <c r="AJI74" s="11"/>
+      <c r="AJJ74" s="11"/>
+      <c r="AJK74" s="11"/>
+      <c r="AJL74" s="11"/>
+      <c r="AJM74" s="11"/>
+      <c r="AJN74" s="11"/>
+      <c r="AJO74" s="11"/>
+      <c r="AJP74" s="11"/>
+      <c r="AJQ74" s="11"/>
+      <c r="AJR74" s="11"/>
+      <c r="AJS74" s="11"/>
+      <c r="AJT74" s="11"/>
+      <c r="AJU74" s="11"/>
+      <c r="AJV74" s="11"/>
+      <c r="AJW74" s="11"/>
+      <c r="AJX74" s="11"/>
+      <c r="AJY74" s="11"/>
+      <c r="AJZ74" s="11"/>
+      <c r="AKA74" s="11"/>
+      <c r="AKB74" s="11"/>
+      <c r="AKC74" s="11"/>
+      <c r="AKD74" s="11"/>
+      <c r="AKE74" s="11"/>
+      <c r="AKF74" s="11"/>
+      <c r="AKG74" s="11"/>
+      <c r="AKH74" s="11"/>
+      <c r="AKI74" s="11"/>
+      <c r="AKJ74" s="11"/>
+      <c r="AKK74" s="11"/>
+      <c r="AKL74" s="11"/>
+      <c r="AKM74" s="11"/>
+      <c r="AKN74" s="11"/>
+      <c r="AKO74" s="11"/>
+      <c r="AKP74" s="11"/>
+      <c r="AKQ74" s="11"/>
+      <c r="AKR74" s="11"/>
+      <c r="AKS74" s="11"/>
+      <c r="AKT74" s="11"/>
+      <c r="AKU74" s="11"/>
+      <c r="AKV74" s="11"/>
+      <c r="AKW74" s="11"/>
+      <c r="AKX74" s="11"/>
+      <c r="AKY74" s="11"/>
+      <c r="AKZ74" s="11"/>
+      <c r="ALA74" s="11"/>
+      <c r="ALB74" s="11"/>
+      <c r="ALC74" s="11"/>
+      <c r="ALD74" s="11"/>
+      <c r="ALE74" s="11"/>
+      <c r="ALF74" s="11"/>
+      <c r="ALG74" s="11"/>
+      <c r="ALH74" s="11"/>
+      <c r="ALI74" s="11"/>
+      <c r="ALJ74" s="11"/>
+      <c r="ALK74" s="11"/>
+      <c r="ALL74" s="11"/>
+      <c r="ALM74" s="11"/>
+      <c r="ALN74" s="11"/>
+      <c r="ALO74" s="11"/>
+      <c r="ALP74" s="11"/>
+      <c r="ALQ74" s="11"/>
+      <c r="ALR74" s="11"/>
+      <c r="ALS74" s="11"/>
+      <c r="ALT74" s="11"/>
+      <c r="ALU74" s="11"/>
+      <c r="ALV74" s="11"/>
+      <c r="ALW74" s="11"/>
+      <c r="ALX74" s="11"/>
+      <c r="ALY74" s="11"/>
+      <c r="ALZ74" s="11"/>
+      <c r="AMA74" s="11"/>
+      <c r="AMB74" s="11"/>
+      <c r="AMC74" s="11"/>
+      <c r="AMD74" s="11"/>
+      <c r="AME74" s="11"/>
+      <c r="AMF74" s="11"/>
+      <c r="AMG74" s="11"/>
+      <c r="AMH74" s="11"/>
+      <c r="AMI74" s="11"/>
+      <c r="AMJ74" s="11"/>
+    </row>
     <row r="1048418" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048419" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048420" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
feat: replace IO2 with VDRIVE_SEN
</commit_message>
<xml_diff>
--- a/bom.xlsx
+++ b/bom.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -134,7 +134,7 @@
     <t xml:space="preserve">Your Instructions / Notes</t>
   </si>
   <si>
-    <t xml:space="preserve">C1, C2, C3, C7, C8, C11, C18, C29, C30, C32</t>
+    <t xml:space="preserve">C1,C2,C3,C7,C8,C11,C18,C29,C30,C31</t>
   </si>
   <si>
     <t xml:space="preserve">Samsung Electro-Mechanics</t>
@@ -152,7 +152,7 @@
     <t xml:space="preserve">SMD</t>
   </si>
   <si>
-    <t xml:space="preserve">C4, C6, C19, C21, C22, C25, C26, C34</t>
+    <t xml:space="preserve">C4,C6,C19,C21,C22,C25,C26,C34</t>
   </si>
   <si>
     <t xml:space="preserve">Murata Electronics</t>
@@ -164,7 +164,7 @@
     <t xml:space="preserve">CAP CER 1000PF 100V C0G/NP0 0402</t>
   </si>
   <si>
-    <t xml:space="preserve">C5, C35, C36</t>
+    <t xml:space="preserve">C5,C35,C36</t>
   </si>
   <si>
     <t xml:space="preserve">GCM1555C1H221JA16D</t>
@@ -173,7 +173,7 @@
     <t xml:space="preserve">CAP CER 220PF 50V C0G/NP0 0402</t>
   </si>
   <si>
-    <t xml:space="preserve">C9, C10</t>
+    <t xml:space="preserve">C9,C10</t>
   </si>
   <si>
     <t xml:space="preserve">GCM1555C1H101JA16D</t>
@@ -182,7 +182,7 @@
     <t xml:space="preserve">CAP CER 100PF 50V C0G/NP0 0402</t>
   </si>
   <si>
-    <t xml:space="preserve">C12, C20, C27</t>
+    <t xml:space="preserve">C12,C20,C27</t>
   </si>
   <si>
     <t xml:space="preserve">Cornell Dubilier Knowles</t>
@@ -218,7 +218,7 @@
     <t xml:space="preserve">CAP CER 10UF 50V X7R 1206</t>
   </si>
   <si>
-    <t xml:space="preserve">C15, C16, C17, C23, C24</t>
+    <t xml:space="preserve">C15,C16,C17,C23,C24</t>
   </si>
   <si>
     <t xml:space="preserve">CL31B105KCHVPJE</t>
@@ -236,7 +236,7 @@
     <t xml:space="preserve">CAP CER 4.7UF 50V X7R 1206</t>
   </si>
   <si>
-    <t xml:space="preserve">C31</t>
+    <t xml:space="preserve">C32</t>
   </si>
   <si>
     <t xml:space="preserve">GRT3195C2A103JA02D</t>
@@ -245,7 +245,7 @@
     <t xml:space="preserve">CAP CER 10000PF 100V C0G 1206</t>
   </si>
   <si>
-    <t xml:space="preserve">C33, C37</t>
+    <t xml:space="preserve">C33,C37</t>
   </si>
   <si>
     <t xml:space="preserve">TDK Corporation</t>
@@ -257,7 +257,7 @@
     <t xml:space="preserve">CAP CER 47UF 6.3V X7S 1206</t>
   </si>
   <si>
-    <t xml:space="preserve">D1, D2, D3, D7, D8, D11, D13, D16, D17, D19</t>
+    <t xml:space="preserve">D1,D2,D3,D7,D8,D11,D13,D16,D17,D19</t>
   </si>
   <si>
     <t xml:space="preserve">onsemi</t>
@@ -344,7 +344,7 @@
     <t xml:space="preserve">TVS DIODE 30VWM 47.5VC ESC</t>
   </si>
   <si>
-    <t xml:space="preserve">D14, D15</t>
+    <t xml:space="preserve">D14,D15</t>
   </si>
   <si>
     <t xml:space="preserve">Micro Commercial Co</t>
@@ -440,7 +440,7 @@
     <t xml:space="preserve">0805</t>
   </si>
   <si>
-    <t xml:space="preserve">Q1, Q6</t>
+    <t xml:space="preserve">Q1,Q6</t>
   </si>
   <si>
     <t xml:space="preserve">Rohm Semiconductor</t>
@@ -467,7 +467,7 @@
     <t xml:space="preserve">SOT-363</t>
   </si>
   <si>
-    <t xml:space="preserve">Q3, Q4, Q5, Q7, Q8</t>
+    <t xml:space="preserve">Q3,Q4,Q5,Q7,Q8</t>
   </si>
   <si>
     <t xml:space="preserve">Vishay Siliconix</t>
@@ -485,28 +485,28 @@
     <t xml:space="preserve">Q9</t>
   </si>
   <si>
+    <t xml:space="preserve">ANBON SEMICONDUCTOR (INT'L) LIMITED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BC847B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PLASTIC ENCAPSULATE TRANSISTORS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOT-23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q10</t>
+  </si>
+  <si>
     <t xml:space="preserve">BSS138</t>
   </si>
   <si>
     <t xml:space="preserve">MOSFET N-CH 50V 220MA SOT23-3</t>
   </si>
   <si>
-    <t xml:space="preserve">Q10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ANBON SEMICONDUCTOR (INT'L) LIMITED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BC847B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PLASTIC ENCAPSULATE TRANSISTORS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SOT-23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R1, R8, R18, R20, R34, R35, R36, R43, R48, R50</t>
+    <t xml:space="preserve">R1,R8,R18,R20,R34,R35,R36,R43,R50,R54</t>
   </si>
   <si>
     <t xml:space="preserve">YAGEO</t>
@@ -518,7 +518,7 @@
     <t xml:space="preserve">RES 10K OHM 1% 1/16W 0402</t>
   </si>
   <si>
-    <t xml:space="preserve">R2, R3, R4, R5</t>
+    <t xml:space="preserve">R2,R3,R4,R5</t>
   </si>
   <si>
     <t xml:space="preserve">RC0402FR-0722KL</t>
@@ -527,7 +527,7 @@
     <t xml:space="preserve">RES 22K OHM 1% 1/16W 0402</t>
   </si>
   <si>
-    <t xml:space="preserve">R6, R7, R31, R49</t>
+    <t xml:space="preserve">R6,R7,R31,R51</t>
   </si>
   <si>
     <t xml:space="preserve">RC0402FR-074K7L</t>
@@ -548,7 +548,7 @@
     <t xml:space="preserve">RES SMD 2.2 OHM 1% 1/2W 0805</t>
   </si>
   <si>
-    <t xml:space="preserve">R10, R11, R14, R32, R45, R51</t>
+    <t xml:space="preserve">R10,R11,R14,R32,R45,R55</t>
   </si>
   <si>
     <t xml:space="preserve">RC0402FR-071KL</t>
@@ -557,7 +557,7 @@
     <t xml:space="preserve">RES 1K OHM 1% 1/16W 0402</t>
   </si>
   <si>
-    <t xml:space="preserve">R12, R13, R22, R26, R27</t>
+    <t xml:space="preserve">R12,R13,R22,R26,R27</t>
   </si>
   <si>
     <t xml:space="preserve">RC0402FR-073K3L</t>
@@ -566,7 +566,7 @@
     <t xml:space="preserve">RES 3.3K OHM 1% 1/16W 0402</t>
   </si>
   <si>
-    <t xml:space="preserve">R15, R16, R52, R53</t>
+    <t xml:space="preserve">R15,R16,R52,R53</t>
   </si>
   <si>
     <t xml:space="preserve">RC0402FR-0733RL</t>
@@ -584,7 +584,7 @@
     <t xml:space="preserve">RES 220 OHM 1% 1/16W 0402</t>
   </si>
   <si>
-    <t xml:space="preserve">R19, R54</t>
+    <t xml:space="preserve">R19,R57</t>
   </si>
   <si>
     <t xml:space="preserve">DNP</t>
@@ -608,7 +608,7 @@
     <t xml:space="preserve">RES 562 OHM 1% 1/16W 0402</t>
   </si>
   <si>
-    <t xml:space="preserve">R24, R25</t>
+    <t xml:space="preserve">R24,R25</t>
   </si>
   <si>
     <t xml:space="preserve">R28</t>
@@ -620,7 +620,7 @@
     <t xml:space="preserve">RES 422 OHM 1% 1/16W 0402</t>
   </si>
   <si>
-    <t xml:space="preserve">R29, R30, R46, R47</t>
+    <t xml:space="preserve">R29,R30,R46,R49</t>
   </si>
   <si>
     <t xml:space="preserve">RC0402FR-0747RL</t>
@@ -638,7 +638,7 @@
     <t xml:space="preserve">RES 180 OHM 1% 1/16W 0402</t>
   </si>
   <si>
-    <t xml:space="preserve">R37, R44</t>
+    <t xml:space="preserve">R37,R44,R47</t>
   </si>
   <si>
     <t xml:space="preserve">RC0402FR-0714K3L</t>
@@ -647,7 +647,7 @@
     <t xml:space="preserve">RES 14.3K OHM 1% 1/16W 0402</t>
   </si>
   <si>
-    <t xml:space="preserve">R38</t>
+    <t xml:space="preserve">R38,R48</t>
   </si>
   <si>
     <t xml:space="preserve">RC0402FR-07470RL</t>
@@ -665,7 +665,7 @@
     <t xml:space="preserve">RES 18.7K OHM 1% 1/16W 0402</t>
   </si>
   <si>
-    <t xml:space="preserve">R40, R41</t>
+    <t xml:space="preserve">R40,R41</t>
   </si>
   <si>
     <t xml:space="preserve">RC0402FR-075K1L</t>
@@ -683,7 +683,7 @@
     <t xml:space="preserve">RES 39K OHM 1% 1/16W 0402</t>
   </si>
   <si>
-    <t xml:space="preserve">R55</t>
+    <t xml:space="preserve">R56</t>
   </si>
   <si>
     <t xml:space="preserve">Panasonic Electronic Components</t>
@@ -1105,13 +1105,13 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>649800</xdr:colOff>
+      <xdr:colOff>649080</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>142200</xdr:rowOff>
+      <xdr:rowOff>141480</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="0" name="图片 1" descr="pcbway-400x400.jpg"/>
+        <xdr:cNvPr id="1" name="图片 1" descr="pcbway-400x400.jpg"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1121,7 +1121,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="9360" y="211680"/>
-          <a:ext cx="1360440" cy="359280"/>
+          <a:ext cx="1359720" cy="358560"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1145,37 +1145,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18a303"/>
+        <a:srgbClr val="18A303"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369a3"/>
+        <a:srgbClr val="0369A3"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="a33e03"/>
+        <a:srgbClr val="A33E03"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8e03a3"/>
+        <a:srgbClr val="8E03A3"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="c99c00"/>
+        <a:srgbClr val="C99C00"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="c9211e"/>
+        <a:srgbClr val="C9211E"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ee"/>
+        <a:srgbClr val="0000EE"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551a8b"/>
+        <a:srgbClr val="551A8B"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -2097,48 +2097,1063 @@
         <v>1</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>52</v>
+        <v>127</v>
       </c>
       <c r="E36" s="7" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G36" s="9" t="s">
-        <v>70</v>
+        <v>130</v>
       </c>
       <c r="H36" s="10" t="s">
         <v>15</v>
       </c>
       <c r="I36" s="10"/>
     </row>
-    <row r="37" s="11" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="6" t="n">
         <v>31</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C37" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>130</v>
+        <v>52</v>
       </c>
       <c r="E37" s="7" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G37" s="9" t="s">
-        <v>133</v>
+        <v>70</v>
       </c>
       <c r="H37" s="10" t="s">
         <v>15</v>
       </c>
       <c r="I37" s="10"/>
+      <c r="J37" s="11"/>
+      <c r="K37" s="11"/>
+      <c r="L37" s="11"/>
+      <c r="M37" s="11"/>
+      <c r="N37" s="11"/>
+      <c r="O37" s="11"/>
+      <c r="P37" s="11"/>
+      <c r="Q37" s="11"/>
+      <c r="R37" s="11"/>
+      <c r="S37" s="11"/>
+      <c r="T37" s="11"/>
+      <c r="U37" s="11"/>
+      <c r="V37" s="11"/>
+      <c r="W37" s="11"/>
+      <c r="X37" s="11"/>
+      <c r="Y37" s="11"/>
+      <c r="Z37" s="11"/>
+      <c r="AA37" s="11"/>
+      <c r="AB37" s="11"/>
+      <c r="AC37" s="11"/>
+      <c r="AD37" s="11"/>
+      <c r="AE37" s="11"/>
+      <c r="AF37" s="11"/>
+      <c r="AG37" s="11"/>
+      <c r="AH37" s="11"/>
+      <c r="AI37" s="11"/>
+      <c r="AJ37" s="11"/>
+      <c r="AK37" s="11"/>
+      <c r="AL37" s="11"/>
+      <c r="AM37" s="11"/>
+      <c r="AN37" s="11"/>
+      <c r="AO37" s="11"/>
+      <c r="AP37" s="11"/>
+      <c r="AQ37" s="11"/>
+      <c r="AR37" s="11"/>
+      <c r="AS37" s="11"/>
+      <c r="AT37" s="11"/>
+      <c r="AU37" s="11"/>
+      <c r="AV37" s="11"/>
+      <c r="AW37" s="11"/>
+      <c r="AX37" s="11"/>
+      <c r="AY37" s="11"/>
+      <c r="AZ37" s="11"/>
+      <c r="BA37" s="11"/>
+      <c r="BB37" s="11"/>
+      <c r="BC37" s="11"/>
+      <c r="BD37" s="11"/>
+      <c r="BE37" s="11"/>
+      <c r="BF37" s="11"/>
+      <c r="BG37" s="11"/>
+      <c r="BH37" s="11"/>
+      <c r="BI37" s="11"/>
+      <c r="BJ37" s="11"/>
+      <c r="BK37" s="11"/>
+      <c r="BL37" s="11"/>
+      <c r="BM37" s="11"/>
+      <c r="BN37" s="11"/>
+      <c r="BO37" s="11"/>
+      <c r="BP37" s="11"/>
+      <c r="BQ37" s="11"/>
+      <c r="BR37" s="11"/>
+      <c r="BS37" s="11"/>
+      <c r="BT37" s="11"/>
+      <c r="BU37" s="11"/>
+      <c r="BV37" s="11"/>
+      <c r="BW37" s="11"/>
+      <c r="BX37" s="11"/>
+      <c r="BY37" s="11"/>
+      <c r="BZ37" s="11"/>
+      <c r="CA37" s="11"/>
+      <c r="CB37" s="11"/>
+      <c r="CC37" s="11"/>
+      <c r="CD37" s="11"/>
+      <c r="CE37" s="11"/>
+      <c r="CF37" s="11"/>
+      <c r="CG37" s="11"/>
+      <c r="CH37" s="11"/>
+      <c r="CI37" s="11"/>
+      <c r="CJ37" s="11"/>
+      <c r="CK37" s="11"/>
+      <c r="CL37" s="11"/>
+      <c r="CM37" s="11"/>
+      <c r="CN37" s="11"/>
+      <c r="CO37" s="11"/>
+      <c r="CP37" s="11"/>
+      <c r="CQ37" s="11"/>
+      <c r="CR37" s="11"/>
+      <c r="CS37" s="11"/>
+      <c r="CT37" s="11"/>
+      <c r="CU37" s="11"/>
+      <c r="CV37" s="11"/>
+      <c r="CW37" s="11"/>
+      <c r="CX37" s="11"/>
+      <c r="CY37" s="11"/>
+      <c r="CZ37" s="11"/>
+      <c r="DA37" s="11"/>
+      <c r="DB37" s="11"/>
+      <c r="DC37" s="11"/>
+      <c r="DD37" s="11"/>
+      <c r="DE37" s="11"/>
+      <c r="DF37" s="11"/>
+      <c r="DG37" s="11"/>
+      <c r="DH37" s="11"/>
+      <c r="DI37" s="11"/>
+      <c r="DJ37" s="11"/>
+      <c r="DK37" s="11"/>
+      <c r="DL37" s="11"/>
+      <c r="DM37" s="11"/>
+      <c r="DN37" s="11"/>
+      <c r="DO37" s="11"/>
+      <c r="DP37" s="11"/>
+      <c r="DQ37" s="11"/>
+      <c r="DR37" s="11"/>
+      <c r="DS37" s="11"/>
+      <c r="DT37" s="11"/>
+      <c r="DU37" s="11"/>
+      <c r="DV37" s="11"/>
+      <c r="DW37" s="11"/>
+      <c r="DX37" s="11"/>
+      <c r="DY37" s="11"/>
+      <c r="DZ37" s="11"/>
+      <c r="EA37" s="11"/>
+      <c r="EB37" s="11"/>
+      <c r="EC37" s="11"/>
+      <c r="ED37" s="11"/>
+      <c r="EE37" s="11"/>
+      <c r="EF37" s="11"/>
+      <c r="EG37" s="11"/>
+      <c r="EH37" s="11"/>
+      <c r="EI37" s="11"/>
+      <c r="EJ37" s="11"/>
+      <c r="EK37" s="11"/>
+      <c r="EL37" s="11"/>
+      <c r="EM37" s="11"/>
+      <c r="EN37" s="11"/>
+      <c r="EO37" s="11"/>
+      <c r="EP37" s="11"/>
+      <c r="EQ37" s="11"/>
+      <c r="ER37" s="11"/>
+      <c r="ES37" s="11"/>
+      <c r="ET37" s="11"/>
+      <c r="EU37" s="11"/>
+      <c r="EV37" s="11"/>
+      <c r="EW37" s="11"/>
+      <c r="EX37" s="11"/>
+      <c r="EY37" s="11"/>
+      <c r="EZ37" s="11"/>
+      <c r="FA37" s="11"/>
+      <c r="FB37" s="11"/>
+      <c r="FC37" s="11"/>
+      <c r="FD37" s="11"/>
+      <c r="FE37" s="11"/>
+      <c r="FF37" s="11"/>
+      <c r="FG37" s="11"/>
+      <c r="FH37" s="11"/>
+      <c r="FI37" s="11"/>
+      <c r="FJ37" s="11"/>
+      <c r="FK37" s="11"/>
+      <c r="FL37" s="11"/>
+      <c r="FM37" s="11"/>
+      <c r="FN37" s="11"/>
+      <c r="FO37" s="11"/>
+      <c r="FP37" s="11"/>
+      <c r="FQ37" s="11"/>
+      <c r="FR37" s="11"/>
+      <c r="FS37" s="11"/>
+      <c r="FT37" s="11"/>
+      <c r="FU37" s="11"/>
+      <c r="FV37" s="11"/>
+      <c r="FW37" s="11"/>
+      <c r="FX37" s="11"/>
+      <c r="FY37" s="11"/>
+      <c r="FZ37" s="11"/>
+      <c r="GA37" s="11"/>
+      <c r="GB37" s="11"/>
+      <c r="GC37" s="11"/>
+      <c r="GD37" s="11"/>
+      <c r="GE37" s="11"/>
+      <c r="GF37" s="11"/>
+      <c r="GG37" s="11"/>
+      <c r="GH37" s="11"/>
+      <c r="GI37" s="11"/>
+      <c r="GJ37" s="11"/>
+      <c r="GK37" s="11"/>
+      <c r="GL37" s="11"/>
+      <c r="GM37" s="11"/>
+      <c r="GN37" s="11"/>
+      <c r="GO37" s="11"/>
+      <c r="GP37" s="11"/>
+      <c r="GQ37" s="11"/>
+      <c r="GR37" s="11"/>
+      <c r="GS37" s="11"/>
+      <c r="GT37" s="11"/>
+      <c r="GU37" s="11"/>
+      <c r="GV37" s="11"/>
+      <c r="GW37" s="11"/>
+      <c r="GX37" s="11"/>
+      <c r="GY37" s="11"/>
+      <c r="GZ37" s="11"/>
+      <c r="HA37" s="11"/>
+      <c r="HB37" s="11"/>
+      <c r="HC37" s="11"/>
+      <c r="HD37" s="11"/>
+      <c r="HE37" s="11"/>
+      <c r="HF37" s="11"/>
+      <c r="HG37" s="11"/>
+      <c r="HH37" s="11"/>
+      <c r="HI37" s="11"/>
+      <c r="HJ37" s="11"/>
+      <c r="HK37" s="11"/>
+      <c r="HL37" s="11"/>
+      <c r="HM37" s="11"/>
+      <c r="HN37" s="11"/>
+      <c r="HO37" s="11"/>
+      <c r="HP37" s="11"/>
+      <c r="HQ37" s="11"/>
+      <c r="HR37" s="11"/>
+      <c r="HS37" s="11"/>
+      <c r="HT37" s="11"/>
+      <c r="HU37" s="11"/>
+      <c r="HV37" s="11"/>
+      <c r="HW37" s="11"/>
+      <c r="HX37" s="11"/>
+      <c r="HY37" s="11"/>
+      <c r="HZ37" s="11"/>
+      <c r="IA37" s="11"/>
+      <c r="IB37" s="11"/>
+      <c r="IC37" s="11"/>
+      <c r="ID37" s="11"/>
+      <c r="IE37" s="11"/>
+      <c r="IF37" s="11"/>
+      <c r="IG37" s="11"/>
+      <c r="IH37" s="11"/>
+      <c r="II37" s="11"/>
+      <c r="IJ37" s="11"/>
+      <c r="IK37" s="11"/>
+      <c r="IL37" s="11"/>
+      <c r="IM37" s="11"/>
+      <c r="IN37" s="11"/>
+      <c r="IO37" s="11"/>
+      <c r="IP37" s="11"/>
+      <c r="IQ37" s="11"/>
+      <c r="IR37" s="11"/>
+      <c r="IS37" s="11"/>
+      <c r="IT37" s="11"/>
+      <c r="IU37" s="11"/>
+      <c r="IV37" s="11"/>
+      <c r="IW37" s="11"/>
+      <c r="IX37" s="11"/>
+      <c r="IY37" s="11"/>
+      <c r="IZ37" s="11"/>
+      <c r="JA37" s="11"/>
+      <c r="JB37" s="11"/>
+      <c r="JC37" s="11"/>
+      <c r="JD37" s="11"/>
+      <c r="JE37" s="11"/>
+      <c r="JF37" s="11"/>
+      <c r="JG37" s="11"/>
+      <c r="JH37" s="11"/>
+      <c r="JI37" s="11"/>
+      <c r="JJ37" s="11"/>
+      <c r="JK37" s="11"/>
+      <c r="JL37" s="11"/>
+      <c r="JM37" s="11"/>
+      <c r="JN37" s="11"/>
+      <c r="JO37" s="11"/>
+      <c r="JP37" s="11"/>
+      <c r="JQ37" s="11"/>
+      <c r="JR37" s="11"/>
+      <c r="JS37" s="11"/>
+      <c r="JT37" s="11"/>
+      <c r="JU37" s="11"/>
+      <c r="JV37" s="11"/>
+      <c r="JW37" s="11"/>
+      <c r="JX37" s="11"/>
+      <c r="JY37" s="11"/>
+      <c r="JZ37" s="11"/>
+      <c r="KA37" s="11"/>
+      <c r="KB37" s="11"/>
+      <c r="KC37" s="11"/>
+      <c r="KD37" s="11"/>
+      <c r="KE37" s="11"/>
+      <c r="KF37" s="11"/>
+      <c r="KG37" s="11"/>
+      <c r="KH37" s="11"/>
+      <c r="KI37" s="11"/>
+      <c r="KJ37" s="11"/>
+      <c r="KK37" s="11"/>
+      <c r="KL37" s="11"/>
+      <c r="KM37" s="11"/>
+      <c r="KN37" s="11"/>
+      <c r="KO37" s="11"/>
+      <c r="KP37" s="11"/>
+      <c r="KQ37" s="11"/>
+      <c r="KR37" s="11"/>
+      <c r="KS37" s="11"/>
+      <c r="KT37" s="11"/>
+      <c r="KU37" s="11"/>
+      <c r="KV37" s="11"/>
+      <c r="KW37" s="11"/>
+      <c r="KX37" s="11"/>
+      <c r="KY37" s="11"/>
+      <c r="KZ37" s="11"/>
+      <c r="LA37" s="11"/>
+      <c r="LB37" s="11"/>
+      <c r="LC37" s="11"/>
+      <c r="LD37" s="11"/>
+      <c r="LE37" s="11"/>
+      <c r="LF37" s="11"/>
+      <c r="LG37" s="11"/>
+      <c r="LH37" s="11"/>
+      <c r="LI37" s="11"/>
+      <c r="LJ37" s="11"/>
+      <c r="LK37" s="11"/>
+      <c r="LL37" s="11"/>
+      <c r="LM37" s="11"/>
+      <c r="LN37" s="11"/>
+      <c r="LO37" s="11"/>
+      <c r="LP37" s="11"/>
+      <c r="LQ37" s="11"/>
+      <c r="LR37" s="11"/>
+      <c r="LS37" s="11"/>
+      <c r="LT37" s="11"/>
+      <c r="LU37" s="11"/>
+      <c r="LV37" s="11"/>
+      <c r="LW37" s="11"/>
+      <c r="LX37" s="11"/>
+      <c r="LY37" s="11"/>
+      <c r="LZ37" s="11"/>
+      <c r="MA37" s="11"/>
+      <c r="MB37" s="11"/>
+      <c r="MC37" s="11"/>
+      <c r="MD37" s="11"/>
+      <c r="ME37" s="11"/>
+      <c r="MF37" s="11"/>
+      <c r="MG37" s="11"/>
+      <c r="MH37" s="11"/>
+      <c r="MI37" s="11"/>
+      <c r="MJ37" s="11"/>
+      <c r="MK37" s="11"/>
+      <c r="ML37" s="11"/>
+      <c r="MM37" s="11"/>
+      <c r="MN37" s="11"/>
+      <c r="MO37" s="11"/>
+      <c r="MP37" s="11"/>
+      <c r="MQ37" s="11"/>
+      <c r="MR37" s="11"/>
+      <c r="MS37" s="11"/>
+      <c r="MT37" s="11"/>
+      <c r="MU37" s="11"/>
+      <c r="MV37" s="11"/>
+      <c r="MW37" s="11"/>
+      <c r="MX37" s="11"/>
+      <c r="MY37" s="11"/>
+      <c r="MZ37" s="11"/>
+      <c r="NA37" s="11"/>
+      <c r="NB37" s="11"/>
+      <c r="NC37" s="11"/>
+      <c r="ND37" s="11"/>
+      <c r="NE37" s="11"/>
+      <c r="NF37" s="11"/>
+      <c r="NG37" s="11"/>
+      <c r="NH37" s="11"/>
+      <c r="NI37" s="11"/>
+      <c r="NJ37" s="11"/>
+      <c r="NK37" s="11"/>
+      <c r="NL37" s="11"/>
+      <c r="NM37" s="11"/>
+      <c r="NN37" s="11"/>
+      <c r="NO37" s="11"/>
+      <c r="NP37" s="11"/>
+      <c r="NQ37" s="11"/>
+      <c r="NR37" s="11"/>
+      <c r="NS37" s="11"/>
+      <c r="NT37" s="11"/>
+      <c r="NU37" s="11"/>
+      <c r="NV37" s="11"/>
+      <c r="NW37" s="11"/>
+      <c r="NX37" s="11"/>
+      <c r="NY37" s="11"/>
+      <c r="NZ37" s="11"/>
+      <c r="OA37" s="11"/>
+      <c r="OB37" s="11"/>
+      <c r="OC37" s="11"/>
+      <c r="OD37" s="11"/>
+      <c r="OE37" s="11"/>
+      <c r="OF37" s="11"/>
+      <c r="OG37" s="11"/>
+      <c r="OH37" s="11"/>
+      <c r="OI37" s="11"/>
+      <c r="OJ37" s="11"/>
+      <c r="OK37" s="11"/>
+      <c r="OL37" s="11"/>
+      <c r="OM37" s="11"/>
+      <c r="ON37" s="11"/>
+      <c r="OO37" s="11"/>
+      <c r="OP37" s="11"/>
+      <c r="OQ37" s="11"/>
+      <c r="OR37" s="11"/>
+      <c r="OS37" s="11"/>
+      <c r="OT37" s="11"/>
+      <c r="OU37" s="11"/>
+      <c r="OV37" s="11"/>
+      <c r="OW37" s="11"/>
+      <c r="OX37" s="11"/>
+      <c r="OY37" s="11"/>
+      <c r="OZ37" s="11"/>
+      <c r="PA37" s="11"/>
+      <c r="PB37" s="11"/>
+      <c r="PC37" s="11"/>
+      <c r="PD37" s="11"/>
+      <c r="PE37" s="11"/>
+      <c r="PF37" s="11"/>
+      <c r="PG37" s="11"/>
+      <c r="PH37" s="11"/>
+      <c r="PI37" s="11"/>
+      <c r="PJ37" s="11"/>
+      <c r="PK37" s="11"/>
+      <c r="PL37" s="11"/>
+      <c r="PM37" s="11"/>
+      <c r="PN37" s="11"/>
+      <c r="PO37" s="11"/>
+      <c r="PP37" s="11"/>
+      <c r="PQ37" s="11"/>
+      <c r="PR37" s="11"/>
+      <c r="PS37" s="11"/>
+      <c r="PT37" s="11"/>
+      <c r="PU37" s="11"/>
+      <c r="PV37" s="11"/>
+      <c r="PW37" s="11"/>
+      <c r="PX37" s="11"/>
+      <c r="PY37" s="11"/>
+      <c r="PZ37" s="11"/>
+      <c r="QA37" s="11"/>
+      <c r="QB37" s="11"/>
+      <c r="QC37" s="11"/>
+      <c r="QD37" s="11"/>
+      <c r="QE37" s="11"/>
+      <c r="QF37" s="11"/>
+      <c r="QG37" s="11"/>
+      <c r="QH37" s="11"/>
+      <c r="QI37" s="11"/>
+      <c r="QJ37" s="11"/>
+      <c r="QK37" s="11"/>
+      <c r="QL37" s="11"/>
+      <c r="QM37" s="11"/>
+      <c r="QN37" s="11"/>
+      <c r="QO37" s="11"/>
+      <c r="QP37" s="11"/>
+      <c r="QQ37" s="11"/>
+      <c r="QR37" s="11"/>
+      <c r="QS37" s="11"/>
+      <c r="QT37" s="11"/>
+      <c r="QU37" s="11"/>
+      <c r="QV37" s="11"/>
+      <c r="QW37" s="11"/>
+      <c r="QX37" s="11"/>
+      <c r="QY37" s="11"/>
+      <c r="QZ37" s="11"/>
+      <c r="RA37" s="11"/>
+      <c r="RB37" s="11"/>
+      <c r="RC37" s="11"/>
+      <c r="RD37" s="11"/>
+      <c r="RE37" s="11"/>
+      <c r="RF37" s="11"/>
+      <c r="RG37" s="11"/>
+      <c r="RH37" s="11"/>
+      <c r="RI37" s="11"/>
+      <c r="RJ37" s="11"/>
+      <c r="RK37" s="11"/>
+      <c r="RL37" s="11"/>
+      <c r="RM37" s="11"/>
+      <c r="RN37" s="11"/>
+      <c r="RO37" s="11"/>
+      <c r="RP37" s="11"/>
+      <c r="RQ37" s="11"/>
+      <c r="RR37" s="11"/>
+      <c r="RS37" s="11"/>
+      <c r="RT37" s="11"/>
+      <c r="RU37" s="11"/>
+      <c r="RV37" s="11"/>
+      <c r="RW37" s="11"/>
+      <c r="RX37" s="11"/>
+      <c r="RY37" s="11"/>
+      <c r="RZ37" s="11"/>
+      <c r="SA37" s="11"/>
+      <c r="SB37" s="11"/>
+      <c r="SC37" s="11"/>
+      <c r="SD37" s="11"/>
+      <c r="SE37" s="11"/>
+      <c r="SF37" s="11"/>
+      <c r="SG37" s="11"/>
+      <c r="SH37" s="11"/>
+      <c r="SI37" s="11"/>
+      <c r="SJ37" s="11"/>
+      <c r="SK37" s="11"/>
+      <c r="SL37" s="11"/>
+      <c r="SM37" s="11"/>
+      <c r="SN37" s="11"/>
+      <c r="SO37" s="11"/>
+      <c r="SP37" s="11"/>
+      <c r="SQ37" s="11"/>
+      <c r="SR37" s="11"/>
+      <c r="SS37" s="11"/>
+      <c r="ST37" s="11"/>
+      <c r="SU37" s="11"/>
+      <c r="SV37" s="11"/>
+      <c r="SW37" s="11"/>
+      <c r="SX37" s="11"/>
+      <c r="SY37" s="11"/>
+      <c r="SZ37" s="11"/>
+      <c r="TA37" s="11"/>
+      <c r="TB37" s="11"/>
+      <c r="TC37" s="11"/>
+      <c r="TD37" s="11"/>
+      <c r="TE37" s="11"/>
+      <c r="TF37" s="11"/>
+      <c r="TG37" s="11"/>
+      <c r="TH37" s="11"/>
+      <c r="TI37" s="11"/>
+      <c r="TJ37" s="11"/>
+      <c r="TK37" s="11"/>
+      <c r="TL37" s="11"/>
+      <c r="TM37" s="11"/>
+      <c r="TN37" s="11"/>
+      <c r="TO37" s="11"/>
+      <c r="TP37" s="11"/>
+      <c r="TQ37" s="11"/>
+      <c r="TR37" s="11"/>
+      <c r="TS37" s="11"/>
+      <c r="TT37" s="11"/>
+      <c r="TU37" s="11"/>
+      <c r="TV37" s="11"/>
+      <c r="TW37" s="11"/>
+      <c r="TX37" s="11"/>
+      <c r="TY37" s="11"/>
+      <c r="TZ37" s="11"/>
+      <c r="UA37" s="11"/>
+      <c r="UB37" s="11"/>
+      <c r="UC37" s="11"/>
+      <c r="UD37" s="11"/>
+      <c r="UE37" s="11"/>
+      <c r="UF37" s="11"/>
+      <c r="UG37" s="11"/>
+      <c r="UH37" s="11"/>
+      <c r="UI37" s="11"/>
+      <c r="UJ37" s="11"/>
+      <c r="UK37" s="11"/>
+      <c r="UL37" s="11"/>
+      <c r="UM37" s="11"/>
+      <c r="UN37" s="11"/>
+      <c r="UO37" s="11"/>
+      <c r="UP37" s="11"/>
+      <c r="UQ37" s="11"/>
+      <c r="UR37" s="11"/>
+      <c r="US37" s="11"/>
+      <c r="UT37" s="11"/>
+      <c r="UU37" s="11"/>
+      <c r="UV37" s="11"/>
+      <c r="UW37" s="11"/>
+      <c r="UX37" s="11"/>
+      <c r="UY37" s="11"/>
+      <c r="UZ37" s="11"/>
+      <c r="VA37" s="11"/>
+      <c r="VB37" s="11"/>
+      <c r="VC37" s="11"/>
+      <c r="VD37" s="11"/>
+      <c r="VE37" s="11"/>
+      <c r="VF37" s="11"/>
+      <c r="VG37" s="11"/>
+      <c r="VH37" s="11"/>
+      <c r="VI37" s="11"/>
+      <c r="VJ37" s="11"/>
+      <c r="VK37" s="11"/>
+      <c r="VL37" s="11"/>
+      <c r="VM37" s="11"/>
+      <c r="VN37" s="11"/>
+      <c r="VO37" s="11"/>
+      <c r="VP37" s="11"/>
+      <c r="VQ37" s="11"/>
+      <c r="VR37" s="11"/>
+      <c r="VS37" s="11"/>
+      <c r="VT37" s="11"/>
+      <c r="VU37" s="11"/>
+      <c r="VV37" s="11"/>
+      <c r="VW37" s="11"/>
+      <c r="VX37" s="11"/>
+      <c r="VY37" s="11"/>
+      <c r="VZ37" s="11"/>
+      <c r="WA37" s="11"/>
+      <c r="WB37" s="11"/>
+      <c r="WC37" s="11"/>
+      <c r="WD37" s="11"/>
+      <c r="WE37" s="11"/>
+      <c r="WF37" s="11"/>
+      <c r="WG37" s="11"/>
+      <c r="WH37" s="11"/>
+      <c r="WI37" s="11"/>
+      <c r="WJ37" s="11"/>
+      <c r="WK37" s="11"/>
+      <c r="WL37" s="11"/>
+      <c r="WM37" s="11"/>
+      <c r="WN37" s="11"/>
+      <c r="WO37" s="11"/>
+      <c r="WP37" s="11"/>
+      <c r="WQ37" s="11"/>
+      <c r="WR37" s="11"/>
+      <c r="WS37" s="11"/>
+      <c r="WT37" s="11"/>
+      <c r="WU37" s="11"/>
+      <c r="WV37" s="11"/>
+      <c r="WW37" s="11"/>
+      <c r="WX37" s="11"/>
+      <c r="WY37" s="11"/>
+      <c r="WZ37" s="11"/>
+      <c r="XA37" s="11"/>
+      <c r="XB37" s="11"/>
+      <c r="XC37" s="11"/>
+      <c r="XD37" s="11"/>
+      <c r="XE37" s="11"/>
+      <c r="XF37" s="11"/>
+      <c r="XG37" s="11"/>
+      <c r="XH37" s="11"/>
+      <c r="XI37" s="11"/>
+      <c r="XJ37" s="11"/>
+      <c r="XK37" s="11"/>
+      <c r="XL37" s="11"/>
+      <c r="XM37" s="11"/>
+      <c r="XN37" s="11"/>
+      <c r="XO37" s="11"/>
+      <c r="XP37" s="11"/>
+      <c r="XQ37" s="11"/>
+      <c r="XR37" s="11"/>
+      <c r="XS37" s="11"/>
+      <c r="XT37" s="11"/>
+      <c r="XU37" s="11"/>
+      <c r="XV37" s="11"/>
+      <c r="XW37" s="11"/>
+      <c r="XX37" s="11"/>
+      <c r="XY37" s="11"/>
+      <c r="XZ37" s="11"/>
+      <c r="YA37" s="11"/>
+      <c r="YB37" s="11"/>
+      <c r="YC37" s="11"/>
+      <c r="YD37" s="11"/>
+      <c r="YE37" s="11"/>
+      <c r="YF37" s="11"/>
+      <c r="YG37" s="11"/>
+      <c r="YH37" s="11"/>
+      <c r="YI37" s="11"/>
+      <c r="YJ37" s="11"/>
+      <c r="YK37" s="11"/>
+      <c r="YL37" s="11"/>
+      <c r="YM37" s="11"/>
+      <c r="YN37" s="11"/>
+      <c r="YO37" s="11"/>
+      <c r="YP37" s="11"/>
+      <c r="YQ37" s="11"/>
+      <c r="YR37" s="11"/>
+      <c r="YS37" s="11"/>
+      <c r="YT37" s="11"/>
+      <c r="YU37" s="11"/>
+      <c r="YV37" s="11"/>
+      <c r="YW37" s="11"/>
+      <c r="YX37" s="11"/>
+      <c r="YY37" s="11"/>
+      <c r="YZ37" s="11"/>
+      <c r="ZA37" s="11"/>
+      <c r="ZB37" s="11"/>
+      <c r="ZC37" s="11"/>
+      <c r="ZD37" s="11"/>
+      <c r="ZE37" s="11"/>
+      <c r="ZF37" s="11"/>
+      <c r="ZG37" s="11"/>
+      <c r="ZH37" s="11"/>
+      <c r="ZI37" s="11"/>
+      <c r="ZJ37" s="11"/>
+      <c r="ZK37" s="11"/>
+      <c r="ZL37" s="11"/>
+      <c r="ZM37" s="11"/>
+      <c r="ZN37" s="11"/>
+      <c r="ZO37" s="11"/>
+      <c r="ZP37" s="11"/>
+      <c r="ZQ37" s="11"/>
+      <c r="ZR37" s="11"/>
+      <c r="ZS37" s="11"/>
+      <c r="ZT37" s="11"/>
+      <c r="ZU37" s="11"/>
+      <c r="ZV37" s="11"/>
+      <c r="ZW37" s="11"/>
+      <c r="ZX37" s="11"/>
+      <c r="ZY37" s="11"/>
+      <c r="ZZ37" s="11"/>
+      <c r="AAA37" s="11"/>
+      <c r="AAB37" s="11"/>
+      <c r="AAC37" s="11"/>
+      <c r="AAD37" s="11"/>
+      <c r="AAE37" s="11"/>
+      <c r="AAF37" s="11"/>
+      <c r="AAG37" s="11"/>
+      <c r="AAH37" s="11"/>
+      <c r="AAI37" s="11"/>
+      <c r="AAJ37" s="11"/>
+      <c r="AAK37" s="11"/>
+      <c r="AAL37" s="11"/>
+      <c r="AAM37" s="11"/>
+      <c r="AAN37" s="11"/>
+      <c r="AAO37" s="11"/>
+      <c r="AAP37" s="11"/>
+      <c r="AAQ37" s="11"/>
+      <c r="AAR37" s="11"/>
+      <c r="AAS37" s="11"/>
+      <c r="AAT37" s="11"/>
+      <c r="AAU37" s="11"/>
+      <c r="AAV37" s="11"/>
+      <c r="AAW37" s="11"/>
+      <c r="AAX37" s="11"/>
+      <c r="AAY37" s="11"/>
+      <c r="AAZ37" s="11"/>
+      <c r="ABA37" s="11"/>
+      <c r="ABB37" s="11"/>
+      <c r="ABC37" s="11"/>
+      <c r="ABD37" s="11"/>
+      <c r="ABE37" s="11"/>
+      <c r="ABF37" s="11"/>
+      <c r="ABG37" s="11"/>
+      <c r="ABH37" s="11"/>
+      <c r="ABI37" s="11"/>
+      <c r="ABJ37" s="11"/>
+      <c r="ABK37" s="11"/>
+      <c r="ABL37" s="11"/>
+      <c r="ABM37" s="11"/>
+      <c r="ABN37" s="11"/>
+      <c r="ABO37" s="11"/>
+      <c r="ABP37" s="11"/>
+      <c r="ABQ37" s="11"/>
+      <c r="ABR37" s="11"/>
+      <c r="ABS37" s="11"/>
+      <c r="ABT37" s="11"/>
+      <c r="ABU37" s="11"/>
+      <c r="ABV37" s="11"/>
+      <c r="ABW37" s="11"/>
+      <c r="ABX37" s="11"/>
+      <c r="ABY37" s="11"/>
+      <c r="ABZ37" s="11"/>
+      <c r="ACA37" s="11"/>
+      <c r="ACB37" s="11"/>
+      <c r="ACC37" s="11"/>
+      <c r="ACD37" s="11"/>
+      <c r="ACE37" s="11"/>
+      <c r="ACF37" s="11"/>
+      <c r="ACG37" s="11"/>
+      <c r="ACH37" s="11"/>
+      <c r="ACI37" s="11"/>
+      <c r="ACJ37" s="11"/>
+      <c r="ACK37" s="11"/>
+      <c r="ACL37" s="11"/>
+      <c r="ACM37" s="11"/>
+      <c r="ACN37" s="11"/>
+      <c r="ACO37" s="11"/>
+      <c r="ACP37" s="11"/>
+      <c r="ACQ37" s="11"/>
+      <c r="ACR37" s="11"/>
+      <c r="ACS37" s="11"/>
+      <c r="ACT37" s="11"/>
+      <c r="ACU37" s="11"/>
+      <c r="ACV37" s="11"/>
+      <c r="ACW37" s="11"/>
+      <c r="ACX37" s="11"/>
+      <c r="ACY37" s="11"/>
+      <c r="ACZ37" s="11"/>
+      <c r="ADA37" s="11"/>
+      <c r="ADB37" s="11"/>
+      <c r="ADC37" s="11"/>
+      <c r="ADD37" s="11"/>
+      <c r="ADE37" s="11"/>
+      <c r="ADF37" s="11"/>
+      <c r="ADG37" s="11"/>
+      <c r="ADH37" s="11"/>
+      <c r="ADI37" s="11"/>
+      <c r="ADJ37" s="11"/>
+      <c r="ADK37" s="11"/>
+      <c r="ADL37" s="11"/>
+      <c r="ADM37" s="11"/>
+      <c r="ADN37" s="11"/>
+      <c r="ADO37" s="11"/>
+      <c r="ADP37" s="11"/>
+      <c r="ADQ37" s="11"/>
+      <c r="ADR37" s="11"/>
+      <c r="ADS37" s="11"/>
+      <c r="ADT37" s="11"/>
+      <c r="ADU37" s="11"/>
+      <c r="ADV37" s="11"/>
+      <c r="ADW37" s="11"/>
+      <c r="ADX37" s="11"/>
+      <c r="ADY37" s="11"/>
+      <c r="ADZ37" s="11"/>
+      <c r="AEA37" s="11"/>
+      <c r="AEB37" s="11"/>
+      <c r="AEC37" s="11"/>
+      <c r="AED37" s="11"/>
+      <c r="AEE37" s="11"/>
+      <c r="AEF37" s="11"/>
+      <c r="AEG37" s="11"/>
+      <c r="AEH37" s="11"/>
+      <c r="AEI37" s="11"/>
+      <c r="AEJ37" s="11"/>
+      <c r="AEK37" s="11"/>
+      <c r="AEL37" s="11"/>
+      <c r="AEM37" s="11"/>
+      <c r="AEN37" s="11"/>
+      <c r="AEO37" s="11"/>
+      <c r="AEP37" s="11"/>
+      <c r="AEQ37" s="11"/>
+      <c r="AER37" s="11"/>
+      <c r="AES37" s="11"/>
+      <c r="AET37" s="11"/>
+      <c r="AEU37" s="11"/>
+      <c r="AEV37" s="11"/>
+      <c r="AEW37" s="11"/>
+      <c r="AEX37" s="11"/>
+      <c r="AEY37" s="11"/>
+      <c r="AEZ37" s="11"/>
+      <c r="AFA37" s="11"/>
+      <c r="AFB37" s="11"/>
+      <c r="AFC37" s="11"/>
+      <c r="AFD37" s="11"/>
+      <c r="AFE37" s="11"/>
+      <c r="AFF37" s="11"/>
+      <c r="AFG37" s="11"/>
+      <c r="AFH37" s="11"/>
+      <c r="AFI37" s="11"/>
+      <c r="AFJ37" s="11"/>
+      <c r="AFK37" s="11"/>
+      <c r="AFL37" s="11"/>
+      <c r="AFM37" s="11"/>
+      <c r="AFN37" s="11"/>
+      <c r="AFO37" s="11"/>
+      <c r="AFP37" s="11"/>
+      <c r="AFQ37" s="11"/>
+      <c r="AFR37" s="11"/>
+      <c r="AFS37" s="11"/>
+      <c r="AFT37" s="11"/>
+      <c r="AFU37" s="11"/>
+      <c r="AFV37" s="11"/>
+      <c r="AFW37" s="11"/>
+      <c r="AFX37" s="11"/>
+      <c r="AFY37" s="11"/>
+      <c r="AFZ37" s="11"/>
+      <c r="AGA37" s="11"/>
+      <c r="AGB37" s="11"/>
+      <c r="AGC37" s="11"/>
+      <c r="AGD37" s="11"/>
+      <c r="AGE37" s="11"/>
+      <c r="AGF37" s="11"/>
+      <c r="AGG37" s="11"/>
+      <c r="AGH37" s="11"/>
+      <c r="AGI37" s="11"/>
+      <c r="AGJ37" s="11"/>
+      <c r="AGK37" s="11"/>
+      <c r="AGL37" s="11"/>
+      <c r="AGM37" s="11"/>
+      <c r="AGN37" s="11"/>
+      <c r="AGO37" s="11"/>
+      <c r="AGP37" s="11"/>
+      <c r="AGQ37" s="11"/>
+      <c r="AGR37" s="11"/>
+      <c r="AGS37" s="11"/>
+      <c r="AGT37" s="11"/>
+      <c r="AGU37" s="11"/>
+      <c r="AGV37" s="11"/>
+      <c r="AGW37" s="11"/>
+      <c r="AGX37" s="11"/>
+      <c r="AGY37" s="11"/>
+      <c r="AGZ37" s="11"/>
+      <c r="AHA37" s="11"/>
+      <c r="AHB37" s="11"/>
+      <c r="AHC37" s="11"/>
+      <c r="AHD37" s="11"/>
+      <c r="AHE37" s="11"/>
+      <c r="AHF37" s="11"/>
+      <c r="AHG37" s="11"/>
+      <c r="AHH37" s="11"/>
+      <c r="AHI37" s="11"/>
+      <c r="AHJ37" s="11"/>
+      <c r="AHK37" s="11"/>
+      <c r="AHL37" s="11"/>
+      <c r="AHM37" s="11"/>
+      <c r="AHN37" s="11"/>
+      <c r="AHO37" s="11"/>
+      <c r="AHP37" s="11"/>
+      <c r="AHQ37" s="11"/>
+      <c r="AHR37" s="11"/>
+      <c r="AHS37" s="11"/>
+      <c r="AHT37" s="11"/>
+      <c r="AHU37" s="11"/>
+      <c r="AHV37" s="11"/>
+      <c r="AHW37" s="11"/>
+      <c r="AHX37" s="11"/>
+      <c r="AHY37" s="11"/>
+      <c r="AHZ37" s="11"/>
+      <c r="AIA37" s="11"/>
+      <c r="AIB37" s="11"/>
+      <c r="AIC37" s="11"/>
+      <c r="AID37" s="11"/>
+      <c r="AIE37" s="11"/>
+      <c r="AIF37" s="11"/>
+      <c r="AIG37" s="11"/>
+      <c r="AIH37" s="11"/>
+      <c r="AII37" s="11"/>
+      <c r="AIJ37" s="11"/>
+      <c r="AIK37" s="11"/>
+      <c r="AIL37" s="11"/>
+      <c r="AIM37" s="11"/>
+      <c r="AIN37" s="11"/>
+      <c r="AIO37" s="11"/>
+      <c r="AIP37" s="11"/>
+      <c r="AIQ37" s="11"/>
+      <c r="AIR37" s="11"/>
+      <c r="AIS37" s="11"/>
+      <c r="AIT37" s="11"/>
+      <c r="AIU37" s="11"/>
+      <c r="AIV37" s="11"/>
+      <c r="AIW37" s="11"/>
+      <c r="AIX37" s="11"/>
+      <c r="AIY37" s="11"/>
+      <c r="AIZ37" s="11"/>
+      <c r="AJA37" s="11"/>
+      <c r="AJB37" s="11"/>
+      <c r="AJC37" s="11"/>
+      <c r="AJD37" s="11"/>
+      <c r="AJE37" s="11"/>
+      <c r="AJF37" s="11"/>
+      <c r="AJG37" s="11"/>
+      <c r="AJH37" s="11"/>
+      <c r="AJI37" s="11"/>
+      <c r="AJJ37" s="11"/>
+      <c r="AJK37" s="11"/>
+      <c r="AJL37" s="11"/>
+      <c r="AJM37" s="11"/>
+      <c r="AJN37" s="11"/>
+      <c r="AJO37" s="11"/>
+      <c r="AJP37" s="11"/>
+      <c r="AJQ37" s="11"/>
+      <c r="AJR37" s="11"/>
+      <c r="AJS37" s="11"/>
+      <c r="AJT37" s="11"/>
+      <c r="AJU37" s="11"/>
+      <c r="AJV37" s="11"/>
+      <c r="AJW37" s="11"/>
+      <c r="AJX37" s="11"/>
+      <c r="AJY37" s="11"/>
+      <c r="AJZ37" s="11"/>
+      <c r="AKA37" s="11"/>
+      <c r="AKB37" s="11"/>
+      <c r="AKC37" s="11"/>
+      <c r="AKD37" s="11"/>
+      <c r="AKE37" s="11"/>
+      <c r="AKF37" s="11"/>
+      <c r="AKG37" s="11"/>
+      <c r="AKH37" s="11"/>
+      <c r="AKI37" s="11"/>
+      <c r="AKJ37" s="11"/>
+      <c r="AKK37" s="11"/>
+      <c r="AKL37" s="11"/>
+      <c r="AKM37" s="11"/>
+      <c r="AKN37" s="11"/>
+      <c r="AKO37" s="11"/>
+      <c r="AKP37" s="11"/>
+      <c r="AKQ37" s="11"/>
+      <c r="AKR37" s="11"/>
+      <c r="AKS37" s="11"/>
+      <c r="AKT37" s="11"/>
+      <c r="AKU37" s="11"/>
+      <c r="AKV37" s="11"/>
+      <c r="AKW37" s="11"/>
+      <c r="AKX37" s="11"/>
+      <c r="AKY37" s="11"/>
+      <c r="AKZ37" s="11"/>
+      <c r="ALA37" s="11"/>
+      <c r="ALB37" s="11"/>
+      <c r="ALC37" s="11"/>
+      <c r="ALD37" s="11"/>
+      <c r="ALE37" s="11"/>
+      <c r="ALF37" s="11"/>
+      <c r="ALG37" s="11"/>
+      <c r="ALH37" s="11"/>
+      <c r="ALI37" s="11"/>
+      <c r="ALJ37" s="11"/>
+      <c r="ALK37" s="11"/>
+      <c r="ALL37" s="11"/>
+      <c r="ALM37" s="11"/>
+      <c r="ALN37" s="11"/>
+      <c r="ALO37" s="11"/>
+      <c r="ALP37" s="11"/>
+      <c r="ALQ37" s="11"/>
+      <c r="ALR37" s="11"/>
+      <c r="ALS37" s="11"/>
+      <c r="ALT37" s="11"/>
+      <c r="ALU37" s="11"/>
+      <c r="ALV37" s="11"/>
+      <c r="ALW37" s="11"/>
+      <c r="ALX37" s="11"/>
+      <c r="ALY37" s="11"/>
+      <c r="ALZ37" s="11"/>
+      <c r="AMA37" s="11"/>
+      <c r="AMB37" s="11"/>
+      <c r="AMC37" s="11"/>
+      <c r="AMD37" s="11"/>
+      <c r="AME37" s="11"/>
+      <c r="AMF37" s="11"/>
+      <c r="AMG37" s="11"/>
+      <c r="AMH37" s="11"/>
+      <c r="AMI37" s="11"/>
+      <c r="AMJ37" s="11"/>
     </row>
     <row r="38" s="11" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="6" t="n">
@@ -2541,7 +3556,7 @@
         <v>178</v>
       </c>
       <c r="C53" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D53" s="7" t="s">
         <v>135</v>
@@ -2568,7 +3583,7 @@
         <v>181</v>
       </c>
       <c r="C54" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D54" s="7" t="s">
         <v>135</v>

</xml_diff>

<commit_message>
chore: update BOM (B5819W manufacturer)
</commit_message>
<xml_diff>
--- a/bom.xlsx
+++ b/bom.xlsx
@@ -347,13 +347,13 @@
     <t xml:space="preserve">D14,D15</t>
   </si>
   <si>
-    <t xml:space="preserve">Micro Commercial Co</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B5819W-TP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIODE SCHOTTKY 40V 1A SOD123</t>
+    <t xml:space="preserve">Shenzhen Slkormicro Semicon Co., Ltd.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B5819W</t>
+  </si>
+  <si>
+    <t xml:space="preserve">40V INDEPENDENT TYPE 900MV@3A 1A</t>
   </si>
   <si>
     <t xml:space="preserve">SOD-123</t>
@@ -1105,9 +1105,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>649080</xdr:colOff>
+      <xdr:colOff>648720</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>141480</xdr:rowOff>
+      <xdr:rowOff>141120</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1121,7 +1121,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="9360" y="211680"/>
-          <a:ext cx="1359720" cy="358560"/>
+          <a:ext cx="1359360" cy="358200"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>

<commit_message>
chore: use consistent SOT-23-3 footprint
</commit_message>
<xml_diff>
--- a/bom.xlsx
+++ b/bom.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="242">
   <si>
     <t xml:space="preserve">S3Main PCS BOM</t>
   </si>
@@ -492,9 +492,6 @@
   </si>
   <si>
     <t xml:space="preserve">PLASTIC ENCAPSULATE TRANSISTORS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SOT-23</t>
   </si>
   <si>
     <t xml:space="preserve">Q10</t>
@@ -1105,9 +1102,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>648720</xdr:colOff>
+      <xdr:colOff>648360</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>141120</xdr:rowOff>
+      <xdr:rowOff>140760</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1121,7 +1118,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="9360" y="211680"/>
-          <a:ext cx="1359360" cy="358200"/>
+          <a:ext cx="1359000" cy="357840"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2106,7 +2103,7 @@
         <v>129</v>
       </c>
       <c r="G36" s="9" t="s">
-        <v>130</v>
+        <v>70</v>
       </c>
       <c r="H36" s="10" t="s">
         <v>15</v>
@@ -2118,7 +2115,7 @@
         <v>31</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C37" s="6" t="n">
         <v>1</v>
@@ -2127,10 +2124,10 @@
         <v>52</v>
       </c>
       <c r="E37" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="F37" s="7" t="s">
         <v>132</v>
-      </c>
-      <c r="F37" s="7" t="s">
-        <v>133</v>
       </c>
       <c r="G37" s="9" t="s">
         <v>70</v>
@@ -3160,19 +3157,19 @@
         <v>32</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C38" s="6" t="n">
         <v>10</v>
       </c>
       <c r="D38" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="E38" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="E38" s="7" t="s">
+      <c r="F38" s="7" t="s">
         <v>136</v>
-      </c>
-      <c r="F38" s="7" t="s">
-        <v>137</v>
       </c>
       <c r="G38" s="9" t="s">
         <v>14</v>
@@ -3187,19 +3184,19 @@
         <v>33</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C39" s="6" t="n">
         <v>4</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E39" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="F39" s="7" t="s">
         <v>139</v>
-      </c>
-      <c r="F39" s="7" t="s">
-        <v>140</v>
       </c>
       <c r="G39" s="9" t="s">
         <v>14</v>
@@ -3214,19 +3211,19 @@
         <v>34</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C40" s="6" t="n">
         <v>4</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E40" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="F40" s="7" t="s">
         <v>142</v>
-      </c>
-      <c r="F40" s="7" t="s">
-        <v>143</v>
       </c>
       <c r="G40" s="9" t="s">
         <v>14</v>
@@ -3241,19 +3238,19 @@
         <v>35</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C41" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D41" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="E41" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="E41" s="7" t="s">
+      <c r="F41" s="7" t="s">
         <v>146</v>
-      </c>
-      <c r="F41" s="7" t="s">
-        <v>147</v>
       </c>
       <c r="G41" s="9" t="s">
         <v>111</v>
@@ -3268,19 +3265,19 @@
         <v>36</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C42" s="6" t="n">
         <v>6</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E42" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="F42" s="7" t="s">
         <v>149</v>
-      </c>
-      <c r="F42" s="7" t="s">
-        <v>150</v>
       </c>
       <c r="G42" s="9" t="s">
         <v>14</v>
@@ -3295,19 +3292,19 @@
         <v>37</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C43" s="6" t="n">
         <v>5</v>
       </c>
       <c r="D43" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E43" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="F43" s="7" t="s">
         <v>152</v>
-      </c>
-      <c r="F43" s="7" t="s">
-        <v>153</v>
       </c>
       <c r="G43" s="9" t="s">
         <v>14</v>
@@ -3322,19 +3319,19 @@
         <v>38</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C44" s="6" t="n">
         <v>4</v>
       </c>
       <c r="D44" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E44" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="F44" s="7" t="s">
         <v>155</v>
-      </c>
-      <c r="F44" s="7" t="s">
-        <v>156</v>
       </c>
       <c r="G44" s="9" t="s">
         <v>14</v>
@@ -3349,19 +3346,19 @@
         <v>39</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C45" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D45" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E45" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="F45" s="8" t="s">
         <v>158</v>
-      </c>
-      <c r="F45" s="8" t="s">
-        <v>159</v>
       </c>
       <c r="G45" s="9" t="s">
         <v>14</v>
@@ -3376,7 +3373,7 @@
         <v>40</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C46" s="6" t="n">
         <v>2</v>
@@ -3385,10 +3382,10 @@
       <c r="E46" s="7"/>
       <c r="F46" s="8"/>
       <c r="G46" s="10" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H46" s="10" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="I46" s="10"/>
     </row>
@@ -3397,19 +3394,19 @@
         <v>41</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C47" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E47" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="F47" s="7" t="s">
         <v>163</v>
-      </c>
-      <c r="F47" s="7" t="s">
-        <v>164</v>
       </c>
       <c r="G47" s="9" t="s">
         <v>14</v>
@@ -3424,19 +3421,19 @@
         <v>42</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C48" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D48" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E48" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="F48" s="8" t="s">
         <v>166</v>
-      </c>
-      <c r="F48" s="8" t="s">
-        <v>167</v>
       </c>
       <c r="G48" s="9" t="s">
         <v>14</v>
@@ -3451,7 +3448,7 @@
         <v>43</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C49" s="6" t="n">
         <v>2</v>
@@ -3460,10 +3457,10 @@
       <c r="E49" s="7"/>
       <c r="F49" s="8"/>
       <c r="G49" s="10" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H49" s="10" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="I49" s="10"/>
     </row>
@@ -3472,19 +3469,19 @@
         <v>44</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C50" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D50" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E50" s="7" t="s">
+        <v>169</v>
+      </c>
+      <c r="F50" s="8" t="s">
         <v>170</v>
-      </c>
-      <c r="F50" s="8" t="s">
-        <v>171</v>
       </c>
       <c r="G50" s="9" t="s">
         <v>14</v>
@@ -3499,19 +3496,19 @@
         <v>45</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C51" s="6" t="n">
         <v>4</v>
       </c>
       <c r="D51" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E51" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="F51" s="8" t="s">
         <v>173</v>
-      </c>
-      <c r="F51" s="8" t="s">
-        <v>174</v>
       </c>
       <c r="G51" s="9" t="s">
         <v>14</v>
@@ -3526,19 +3523,19 @@
         <v>46</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C52" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D52" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E52" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="F52" s="8" t="s">
         <v>176</v>
-      </c>
-      <c r="F52" s="8" t="s">
-        <v>177</v>
       </c>
       <c r="G52" s="9" t="s">
         <v>14</v>
@@ -3553,19 +3550,19 @@
         <v>47</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C53" s="6" t="n">
         <v>3</v>
       </c>
       <c r="D53" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E53" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="F53" s="8" t="s">
         <v>179</v>
-      </c>
-      <c r="F53" s="8" t="s">
-        <v>180</v>
       </c>
       <c r="G53" s="9" t="s">
         <v>14</v>
@@ -3580,19 +3577,19 @@
         <v>48</v>
       </c>
       <c r="B54" s="7" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C54" s="6" t="n">
         <v>2</v>
       </c>
       <c r="D54" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E54" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="F54" s="8" t="s">
         <v>182</v>
-      </c>
-      <c r="F54" s="8" t="s">
-        <v>183</v>
       </c>
       <c r="G54" s="9" t="s">
         <v>14</v>
@@ -3607,19 +3604,19 @@
         <v>49</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C55" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D55" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E55" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="F55" s="8" t="s">
         <v>185</v>
-      </c>
-      <c r="F55" s="8" t="s">
-        <v>186</v>
       </c>
       <c r="G55" s="9" t="s">
         <v>14</v>
@@ -3634,19 +3631,19 @@
         <v>50</v>
       </c>
       <c r="B56" s="7" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C56" s="6" t="n">
         <v>2</v>
       </c>
       <c r="D56" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E56" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="F56" s="8" t="s">
         <v>188</v>
-      </c>
-      <c r="F56" s="8" t="s">
-        <v>189</v>
       </c>
       <c r="G56" s="9" t="s">
         <v>14</v>
@@ -3661,19 +3658,19 @@
         <v>51</v>
       </c>
       <c r="B57" s="7" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C57" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D57" s="7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E57" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="F57" s="8" t="s">
         <v>191</v>
-      </c>
-      <c r="F57" s="8" t="s">
-        <v>192</v>
       </c>
       <c r="G57" s="9" t="s">
         <v>14</v>
@@ -3688,19 +3685,19 @@
         <v>52</v>
       </c>
       <c r="B58" s="7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C58" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D58" s="7" t="s">
+        <v>193</v>
+      </c>
+      <c r="E58" s="7" t="s">
         <v>194</v>
       </c>
-      <c r="E58" s="7" t="s">
+      <c r="F58" s="8" t="s">
         <v>195</v>
-      </c>
-      <c r="F58" s="8" t="s">
-        <v>196</v>
       </c>
       <c r="G58" s="9" t="s">
         <v>14</v>
@@ -3715,22 +3712,22 @@
         <v>53</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C59" s="6" t="n">
         <v>2</v>
       </c>
       <c r="D59" s="7" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E59" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="F59" s="8" t="s">
         <v>198</v>
       </c>
-      <c r="F59" s="8" t="s">
+      <c r="G59" s="9" t="s">
         <v>199</v>
-      </c>
-      <c r="G59" s="9" t="s">
-        <v>200</v>
       </c>
       <c r="H59" s="10" t="s">
         <v>15</v>
@@ -3742,7 +3739,7 @@
         <v>54</v>
       </c>
       <c r="B60" s="7" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C60" s="6" t="n">
         <v>1</v>
@@ -3751,13 +3748,13 @@
         <v>52</v>
       </c>
       <c r="E60" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="F60" s="7" t="s">
         <v>202</v>
       </c>
-      <c r="F60" s="7" t="s">
+      <c r="G60" s="9" t="s">
         <v>203</v>
-      </c>
-      <c r="G60" s="9" t="s">
-        <v>204</v>
       </c>
       <c r="H60" s="10" t="s">
         <v>15</v>
@@ -3769,22 +3766,22 @@
         <v>55</v>
       </c>
       <c r="B61" s="7" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C61" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D61" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="E61" s="7" t="s">
         <v>206</v>
       </c>
-      <c r="E61" s="7" t="s">
+      <c r="F61" s="8" t="s">
         <v>207</v>
       </c>
-      <c r="F61" s="8" t="s">
+      <c r="G61" s="9" t="s">
         <v>208</v>
-      </c>
-      <c r="G61" s="9" t="s">
-        <v>209</v>
       </c>
       <c r="H61" s="10" t="s">
         <v>15</v>
@@ -3796,22 +3793,22 @@
         <v>56</v>
       </c>
       <c r="B62" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C62" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D62" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="E62" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="E62" s="7" t="s">
+      <c r="F62" s="8" t="s">
         <v>212</v>
       </c>
-      <c r="F62" s="8" t="s">
+      <c r="G62" s="9" t="s">
         <v>213</v>
-      </c>
-      <c r="G62" s="9" t="s">
-        <v>214</v>
       </c>
       <c r="H62" s="10" t="s">
         <v>15</v>
@@ -3823,19 +3820,19 @@
         <v>57</v>
       </c>
       <c r="B63" s="7" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C63" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D63" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="E63" s="7" t="s">
         <v>216</v>
       </c>
-      <c r="E63" s="7" t="s">
+      <c r="F63" s="8" t="s">
         <v>217</v>
-      </c>
-      <c r="F63" s="8" t="s">
-        <v>218</v>
       </c>
       <c r="G63" s="9"/>
       <c r="H63" s="10" t="s">
@@ -3848,22 +3845,22 @@
         <v>58</v>
       </c>
       <c r="B64" s="7" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C64" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D64" s="7" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E64" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="F64" s="7" t="s">
         <v>220</v>
       </c>
-      <c r="F64" s="7" t="s">
+      <c r="G64" s="9" t="s">
         <v>221</v>
-      </c>
-      <c r="G64" s="9" t="s">
-        <v>222</v>
       </c>
       <c r="H64" s="10" t="s">
         <v>15</v>
@@ -3875,22 +3872,22 @@
         <v>59</v>
       </c>
       <c r="B65" s="7" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C65" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D65" s="7" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E65" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="F65" s="8" t="s">
         <v>224</v>
       </c>
-      <c r="F65" s="8" t="s">
+      <c r="G65" s="9" t="s">
         <v>225</v>
-      </c>
-      <c r="G65" s="9" t="s">
-        <v>226</v>
       </c>
       <c r="H65" s="10" t="s">
         <v>15</v>
@@ -3902,7 +3899,7 @@
         <v>60</v>
       </c>
       <c r="B66" s="7" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C66" s="6" t="n">
         <v>1</v>
@@ -3911,10 +3908,10 @@
         <v>86</v>
       </c>
       <c r="E66" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="F66" s="8" t="s">
         <v>228</v>
-      </c>
-      <c r="F66" s="8" t="s">
-        <v>229</v>
       </c>
       <c r="G66" s="9" t="s">
         <v>75</v>
@@ -3929,22 +3926,22 @@
         <v>61</v>
       </c>
       <c r="B67" s="7" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C67" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D67" s="7" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E67" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="F67" s="12" t="s">
         <v>231</v>
       </c>
-      <c r="F67" s="12" t="s">
+      <c r="G67" s="9" t="s">
         <v>232</v>
-      </c>
-      <c r="G67" s="9" t="s">
-        <v>233</v>
       </c>
       <c r="H67" s="10" t="s">
         <v>15</v>
@@ -3956,7 +3953,7 @@
         <v>62</v>
       </c>
       <c r="B68" s="7" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C68" s="6" t="n">
         <v>1</v>
@@ -3965,13 +3962,13 @@
         <v>86</v>
       </c>
       <c r="E68" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="F68" s="8" t="s">
         <v>235</v>
       </c>
-      <c r="F68" s="8" t="s">
+      <c r="G68" s="9" t="s">
         <v>236</v>
-      </c>
-      <c r="G68" s="9" t="s">
-        <v>237</v>
       </c>
       <c r="H68" s="10" t="s">
         <v>15</v>
@@ -3983,22 +3980,22 @@
         <v>63</v>
       </c>
       <c r="B69" s="7" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C69" s="6" t="n">
         <v>1</v>
       </c>
       <c r="D69" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="E69" s="7" t="s">
         <v>239</v>
       </c>
-      <c r="E69" s="7" t="s">
+      <c r="F69" s="8" t="s">
         <v>240</v>
       </c>
-      <c r="F69" s="8" t="s">
+      <c r="G69" s="9" t="s">
         <v>241</v>
-      </c>
-      <c r="G69" s="9" t="s">
-        <v>242</v>
       </c>
       <c r="H69" s="10" t="s">
         <v>15</v>

</xml_diff>